<commit_message>
segunda atualização do dia
</commit_message>
<xml_diff>
--- a/cypress/downloads/Plataforma externa Volta Redonda.xlsx
+++ b/cypress/downloads/Plataforma externa Volta Redonda.xlsx
@@ -267,101 +267,104 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="65">
-        <v>1706</v>
+      <c t="inlineStr" r="A3">
+        <is>
+          <t xml:space="preserve">dia17</t>
+        </is>
       </c>
       <c r="B3" s="56">
-        <v>0.1</v>
-      </c>
-      <c r="C3" s="65">
-        <v>1706</v>
+        <v>0.5</v>
+      </c>
+      <c t="inlineStr" r="C3">
+        <is>
+          <t xml:space="preserve">dia17</t>
+        </is>
       </c>
       <c t="n" r="D3">
-        <v>10</v>
+        <v>100</v>
       </c>
       <c t="n" r="E3">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c t="inlineStr" r="F3">
         <is>
-          <t xml:space="preserve">17/06/2025 11:00:00</t>
+          <t xml:space="preserve">17/07/2025 08:00:00</t>
         </is>
       </c>
       <c t="inlineStr" r="G3">
         <is>
-          <t xml:space="preserve">17/06/2025 17:00:00</t>
+          <t xml:space="preserve">17/07/2025 19:00:00</t>
         </is>
       </c>
       <c t="inlineStr" r="H3">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">R$ 1.00</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c t="inlineStr" r="A4">
         <is>
-          <t xml:space="preserve">DIA23JUNHO</t>
+          <t xml:space="preserve">teste08/08</t>
         </is>
       </c>
       <c r="B4" s="56">
-        <v>0.5</v>
+        <v>0.1</v>
       </c>
       <c t="inlineStr" r="C4">
         <is>
-          <t xml:space="preserve">DIA23JUNHO</t>
+          <t xml:space="preserve">teste08/08</t>
         </is>
       </c>
       <c t="n" r="D4">
         <v>100</v>
       </c>
       <c t="n" r="E4">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c t="inlineStr" r="F4">
         <is>
-          <t xml:space="preserve">23/06/2025 08:00:00</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c t="inlineStr" r="G4">
         <is>
-          <t xml:space="preserve">30/06/2025 08:00:00</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c t="inlineStr" r="H4">
         <is>
-          <t xml:space="preserve">R$ 1.00</t>
+          <t xml:space="preserve">R$ 10.00</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c t="inlineStr" r="A5">
         <is>
-          <t xml:space="preserve">Teste2306</t>
-        </is>
-      </c>
-      <c r="B5" s="56">
-        <v>0.1</v>
+          <t xml:space="preserve">testecupom</t>
+        </is>
+      </c>
+      <c t="inlineStr" r="B5">
+        <is>
+          <t xml:space="preserve">R$ 10.00</t>
+        </is>
       </c>
       <c t="inlineStr" r="C5">
         <is>
-          <t xml:space="preserve">teste2306</t>
-        </is>
-      </c>
-      <c t="n" r="D5">
-        <v>11</v>
+          <t xml:space="preserve">testecupom</t>
+        </is>
       </c>
       <c t="n" r="E5">
         <v>1</v>
       </c>
       <c t="inlineStr" r="F5">
         <is>
-          <t xml:space="preserve">23/06/2025 15:25:00</t>
+          <t xml:space="preserve">20/08/2025 09:25:00</t>
         </is>
       </c>
       <c t="inlineStr" r="G5">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">22/08/2025 11:30:00</t>
         </is>
       </c>
       <c t="inlineStr" r="H5">
@@ -373,43 +376,40 @@
     <row r="6">
       <c t="inlineStr" r="A6">
         <is>
-          <t xml:space="preserve">dia17</t>
+          <t xml:space="preserve">testecupom21/08</t>
         </is>
       </c>
       <c r="B6" s="56">
-        <v>0.5</v>
+        <v>0.1</v>
       </c>
       <c t="inlineStr" r="C6">
         <is>
-          <t xml:space="preserve">dia17</t>
-        </is>
-      </c>
-      <c t="n" r="D6">
-        <v>100</v>
+          <t xml:space="preserve">testecupom21/08</t>
+        </is>
       </c>
       <c t="n" r="E6">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c t="inlineStr" r="F6">
         <is>
-          <t xml:space="preserve">17/07/2025 08:00:00</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c t="inlineStr" r="G6">
         <is>
-          <t xml:space="preserve">17/07/2025 19:00:00</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c t="inlineStr" r="H6">
         <is>
-          <t xml:space="preserve">R$ 1.00</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c t="inlineStr" r="A7">
         <is>
-          <t xml:space="preserve">teste08/08</t>
+          <t xml:space="preserve">Cupom7</t>
         </is>
       </c>
       <c r="B7" s="56">
@@ -417,14 +417,14 @@
       </c>
       <c t="inlineStr" r="C7">
         <is>
-          <t xml:space="preserve">teste08/08</t>
+          <t xml:space="preserve">0712</t>
         </is>
       </c>
       <c t="n" r="D7">
-        <v>100</v>
+        <v>8</v>
       </c>
       <c t="n" r="E7">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c t="inlineStr" r="F7">
         <is>
@@ -438,37 +438,33 @@
       </c>
       <c t="inlineStr" r="H7">
         <is>
-          <t xml:space="preserve">R$ 10.00</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c t="inlineStr" r="A8">
         <is>
-          <t xml:space="preserve">testecupom</t>
-        </is>
-      </c>
-      <c t="inlineStr" r="B8">
-        <is>
-          <t xml:space="preserve">R$ 10.00</t>
-        </is>
-      </c>
-      <c t="inlineStr" r="C8">
-        <is>
-          <t xml:space="preserve">testecupom</t>
-        </is>
+          <t xml:space="preserve">CUPOM TESTE</t>
+        </is>
+      </c>
+      <c r="B8" s="56">
+        <v>0.5</v>
+      </c>
+      <c r="C8" s="65">
+        <v>1010</v>
       </c>
       <c t="n" r="E8">
         <v>1</v>
       </c>
       <c t="inlineStr" r="F8">
         <is>
-          <t xml:space="preserve">20/08/2025 09:25:00</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c t="inlineStr" r="G8">
         <is>
-          <t xml:space="preserve">22/08/2025 11:30:00</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c t="inlineStr" r="H8">
@@ -480,28 +476,33 @@
     <row r="9">
       <c t="inlineStr" r="A9">
         <is>
-          <t xml:space="preserve">testecupom21/08</t>
-        </is>
-      </c>
-      <c r="B9" s="56">
-        <v>0.1</v>
+          <t xml:space="preserve">Testecupom</t>
+        </is>
+      </c>
+      <c t="inlineStr" r="B9">
+        <is>
+          <t xml:space="preserve">R$ 10.00</t>
+        </is>
       </c>
       <c t="inlineStr" r="C9">
         <is>
-          <t xml:space="preserve">testecupom21/08</t>
-        </is>
+          <t xml:space="preserve">Testecupom</t>
+        </is>
+      </c>
+      <c t="n" r="D9">
+        <v>50</v>
       </c>
       <c t="n" r="E9">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c t="inlineStr" r="F9">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">23/09/2025 08:00:00</t>
         </is>
       </c>
       <c t="inlineStr" r="G9">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">26/09/2025 14:00:00</t>
         </is>
       </c>
       <c t="inlineStr" r="H9">
@@ -513,22 +514,19 @@
     <row r="10">
       <c t="inlineStr" r="A10">
         <is>
-          <t xml:space="preserve">Cupom7</t>
-        </is>
-      </c>
-      <c r="B10" s="56">
-        <v>0.1</v>
-      </c>
-      <c t="inlineStr" r="C10">
-        <is>
-          <t xml:space="preserve">0712</t>
-        </is>
-      </c>
-      <c t="n" r="D10">
-        <v>8</v>
+          <t xml:space="preserve">TESTE</t>
+        </is>
+      </c>
+      <c t="inlineStr" r="B10">
+        <is>
+          <t xml:space="preserve">R$ 60.00</t>
+        </is>
+      </c>
+      <c r="C10" s="65">
+        <v>606060</v>
       </c>
       <c t="n" r="E10">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c t="inlineStr" r="F10">
         <is>
@@ -549,17 +547,17 @@
     <row r="11">
       <c t="inlineStr" r="A11">
         <is>
-          <t xml:space="preserve">CUPOM TESTE</t>
+          <t xml:space="preserve">TESTE</t>
         </is>
       </c>
       <c r="B11" s="56">
         <v>0.5</v>
       </c>
       <c r="C11" s="65">
-        <v>1010</v>
+        <v>505050</v>
       </c>
       <c t="n" r="E11">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c t="inlineStr" r="F11">
         <is>
@@ -580,33 +578,26 @@
     <row r="12">
       <c t="inlineStr" r="A12">
         <is>
-          <t xml:space="preserve">Testecupom</t>
-        </is>
-      </c>
-      <c t="inlineStr" r="B12">
-        <is>
-          <t xml:space="preserve">R$ 10.00</t>
-        </is>
-      </c>
-      <c t="inlineStr" r="C12">
-        <is>
-          <t xml:space="preserve">Testecupom</t>
-        </is>
-      </c>
-      <c t="n" r="D12">
-        <v>50</v>
+          <t xml:space="preserve">teste</t>
+        </is>
+      </c>
+      <c r="B12" s="56">
+        <v>0.5</v>
+      </c>
+      <c r="C12" s="65">
+        <v>4040</v>
       </c>
       <c t="n" r="E12">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c t="inlineStr" r="F12">
         <is>
-          <t xml:space="preserve">23/09/2025 08:00:00</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c t="inlineStr" r="G12">
         <is>
-          <t xml:space="preserve">26/09/2025 14:00:00</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c t="inlineStr" r="H12">
@@ -618,19 +609,24 @@
     <row r="13">
       <c t="inlineStr" r="A13">
         <is>
-          <t xml:space="preserve">TESTE</t>
+          <t xml:space="preserve">teste2609</t>
         </is>
       </c>
       <c t="inlineStr" r="B13">
         <is>
-          <t xml:space="preserve">R$ 60.00</t>
-        </is>
-      </c>
-      <c r="C13" s="65">
-        <v>606060</v>
+          <t xml:space="preserve">R$ 10.00</t>
+        </is>
+      </c>
+      <c t="inlineStr" r="C13">
+        <is>
+          <t xml:space="preserve">teste2609</t>
+        </is>
+      </c>
+      <c t="n" r="D13">
+        <v>100</v>
       </c>
       <c t="n" r="E13">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c t="inlineStr" r="F13">
         <is>
@@ -651,26 +647,33 @@
     <row r="14">
       <c t="inlineStr" r="A14">
         <is>
-          <t xml:space="preserve">TESTE</t>
-        </is>
-      </c>
-      <c r="B14" s="56">
-        <v>0.5</v>
-      </c>
-      <c r="C14" s="65">
-        <v>505050</v>
+          <t xml:space="preserve">testecupom10/10</t>
+        </is>
+      </c>
+      <c t="inlineStr" r="B14">
+        <is>
+          <t xml:space="preserve">R$ 10.00</t>
+        </is>
+      </c>
+      <c t="inlineStr" r="C14">
+        <is>
+          <t xml:space="preserve">testecupom10/10</t>
+        </is>
+      </c>
+      <c t="n" r="D14">
+        <v>100</v>
       </c>
       <c t="n" r="E14">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c t="inlineStr" r="F14">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">10/10/2025 08:00:00</t>
         </is>
       </c>
       <c t="inlineStr" r="G14">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">11/10/2025 14:00:00</t>
         </is>
       </c>
       <c t="inlineStr" r="H14">
@@ -682,17 +685,22 @@
     <row r="15">
       <c t="inlineStr" r="A15">
         <is>
-          <t xml:space="preserve">teste</t>
+          <t xml:space="preserve">cupom14/10</t>
         </is>
       </c>
       <c r="B15" s="56">
-        <v>0.5</v>
-      </c>
-      <c r="C15" s="65">
-        <v>4040</v>
+        <v>0.1</v>
+      </c>
+      <c t="inlineStr" r="C15">
+        <is>
+          <t xml:space="preserve">cupom14/10</t>
+        </is>
+      </c>
+      <c t="n" r="D15">
+        <v>100</v>
       </c>
       <c t="n" r="E15">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c t="inlineStr" r="F15">
         <is>
@@ -713,24 +721,17 @@
     <row r="16">
       <c t="inlineStr" r="A16">
         <is>
-          <t xml:space="preserve">teste2609</t>
-        </is>
-      </c>
-      <c t="inlineStr" r="B16">
-        <is>
-          <t xml:space="preserve">R$ 10.00</t>
-        </is>
-      </c>
-      <c t="inlineStr" r="C16">
-        <is>
-          <t xml:space="preserve">teste2609</t>
-        </is>
-      </c>
-      <c t="n" r="D16">
-        <v>100</v>
+          <t xml:space="preserve">Cupom50</t>
+        </is>
+      </c>
+      <c r="B16" s="56">
+        <v>0.5</v>
+      </c>
+      <c r="C16" s="65">
+        <v>3110</v>
       </c>
       <c t="n" r="E16">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c t="inlineStr" r="F16">
         <is>
@@ -751,91 +752,87 @@
     <row r="17">
       <c t="inlineStr" r="A17">
         <is>
-          <t xml:space="preserve">testecupom10/10</t>
-        </is>
-      </c>
-      <c t="inlineStr" r="B17">
-        <is>
-          <t xml:space="preserve">R$ 10.00</t>
-        </is>
-      </c>
-      <c t="inlineStr" r="C17">
-        <is>
-          <t xml:space="preserve">testecupom10/10</t>
-        </is>
+          <t xml:space="preserve">Teste12/11</t>
+        </is>
+      </c>
+      <c r="B17" s="56">
+        <v>0.5</v>
+      </c>
+      <c r="C17" s="65">
+        <v>105</v>
       </c>
       <c t="n" r="D17">
-        <v>100</v>
+        <v>10</v>
       </c>
       <c t="n" r="E17">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c t="inlineStr" r="F17">
         <is>
-          <t xml:space="preserve">10/10/2025 08:00:00</t>
+          <t xml:space="preserve">12/11/2025 00:00:00</t>
         </is>
       </c>
       <c t="inlineStr" r="G17">
         <is>
-          <t xml:space="preserve">11/10/2025 14:00:00</t>
+          <t xml:space="preserve">01/03/2026 00:00:00</t>
         </is>
       </c>
       <c t="inlineStr" r="H17">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">R$ 1.00</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c t="inlineStr" r="A18">
         <is>
-          <t xml:space="preserve">cupom14/10</t>
-        </is>
-      </c>
-      <c r="B18" s="56">
-        <v>0.1</v>
-      </c>
-      <c t="inlineStr" r="C18">
-        <is>
-          <t xml:space="preserve">cupom14/10</t>
-        </is>
+          <t xml:space="preserve">TESTE12/11</t>
+        </is>
+      </c>
+      <c t="inlineStr" r="B18">
+        <is>
+          <t xml:space="preserve">R$ 1.00</t>
+        </is>
+      </c>
+      <c r="C18" s="65">
+        <v>201</v>
       </c>
       <c t="n" r="D18">
-        <v>100</v>
+        <v>1</v>
       </c>
       <c t="n" r="E18">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c t="inlineStr" r="F18">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">12/11/2025 00:00:00</t>
         </is>
       </c>
       <c t="inlineStr" r="G18">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">01/03/2026 00:00:00</t>
         </is>
       </c>
       <c t="inlineStr" r="H18">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">R$ 1.00</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c t="inlineStr" r="A19">
         <is>
-          <t xml:space="preserve">Cupom50</t>
+          <t xml:space="preserve">cupom502</t>
         </is>
       </c>
       <c r="B19" s="56">
         <v>0.5</v>
       </c>
       <c r="C19" s="65">
-        <v>3110</v>
+        <v>5486</v>
       </c>
       <c t="n" r="E19">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c t="inlineStr" r="F19">
         <is>
@@ -856,20 +853,20 @@
     <row r="20">
       <c t="inlineStr" r="A20">
         <is>
-          <t xml:space="preserve">Teste12/11</t>
+          <t xml:space="preserve">TESTE12/11</t>
         </is>
       </c>
       <c r="B20" s="56">
         <v>0.5</v>
       </c>
       <c r="C20" s="65">
-        <v>105</v>
+        <v>47992458811</v>
       </c>
       <c t="n" r="D20">
-        <v>10</v>
+        <v>100</v>
       </c>
       <c t="n" r="E20">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c t="inlineStr" r="F20">
         <is>
@@ -878,65 +875,68 @@
       </c>
       <c t="inlineStr" r="G20">
         <is>
-          <t xml:space="preserve">01/03/2026 00:00:00</t>
+          <t xml:space="preserve">03/01/2026 07:35:00</t>
         </is>
       </c>
       <c t="inlineStr" r="H20">
         <is>
-          <t xml:space="preserve">R$ 1.00</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c t="inlineStr" r="A21">
         <is>
-          <t xml:space="preserve">TESTE12/11</t>
-        </is>
-      </c>
-      <c t="inlineStr" r="B21">
-        <is>
-          <t xml:space="preserve">R$ 1.00</t>
-        </is>
+          <t xml:space="preserve">Teste</t>
+        </is>
+      </c>
+      <c r="B21" s="56">
+        <v>0.5</v>
       </c>
       <c r="C21" s="65">
-        <v>201</v>
+        <v>1617</v>
       </c>
       <c t="n" r="D21">
-        <v>1</v>
+        <v>100</v>
       </c>
       <c t="n" r="E21">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c t="inlineStr" r="F21">
         <is>
-          <t xml:space="preserve">12/11/2025 00:00:00</t>
+          <t xml:space="preserve">12/11/2025 16:15:00</t>
         </is>
       </c>
       <c t="inlineStr" r="G21">
         <is>
-          <t xml:space="preserve">01/03/2026 00:00:00</t>
+          <t xml:space="preserve">12/11/2025 16:20:00</t>
         </is>
       </c>
       <c t="inlineStr" r="H21">
         <is>
-          <t xml:space="preserve">R$ 1.00</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c t="inlineStr" r="A22">
         <is>
-          <t xml:space="preserve">cupom502</t>
-        </is>
-      </c>
-      <c r="B22" s="56">
-        <v>0.5</v>
+          <t xml:space="preserve">Testeeeee</t>
+        </is>
+      </c>
+      <c t="inlineStr" r="B22">
+        <is>
+          <t xml:space="preserve">R$ 2.00</t>
+        </is>
       </c>
       <c r="C22" s="65">
-        <v>5486</v>
+        <v>2222</v>
+      </c>
+      <c t="n" r="D22">
+        <v>100</v>
       </c>
       <c t="n" r="E22">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c t="inlineStr" r="F22">
         <is>
@@ -957,29 +957,28 @@
     <row r="23">
       <c t="inlineStr" r="A23">
         <is>
-          <t xml:space="preserve">TESTE12/11</t>
+          <t xml:space="preserve">Teste17/11</t>
         </is>
       </c>
       <c r="B23" s="56">
         <v>0.5</v>
       </c>
-      <c r="C23" s="65">
-        <v>47992458811</v>
-      </c>
-      <c t="n" r="D23">
-        <v>100</v>
+      <c t="inlineStr" r="C23">
+        <is>
+          <t xml:space="preserve">Teste17/11</t>
+        </is>
       </c>
       <c t="n" r="E23">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c t="inlineStr" r="F23">
         <is>
-          <t xml:space="preserve">12/11/2025 00:00:00</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c t="inlineStr" r="G23">
         <is>
-          <t xml:space="preserve">03/01/2026 07:35:00</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c t="inlineStr" r="H23">
@@ -991,65 +990,65 @@
     <row r="24">
       <c t="inlineStr" r="A24">
         <is>
-          <t xml:space="preserve">Teste</t>
+          <t xml:space="preserve">teste</t>
         </is>
       </c>
       <c r="B24" s="56">
         <v>0.5</v>
       </c>
       <c r="C24" s="65">
-        <v>1617</v>
+        <v>5050</v>
       </c>
       <c t="n" r="D24">
-        <v>100</v>
+        <v>10</v>
       </c>
       <c t="n" r="E24">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c t="inlineStr" r="F24">
         <is>
-          <t xml:space="preserve">12/11/2025 16:15:00</t>
+          <t xml:space="preserve">21/11/2025 14:55:00</t>
         </is>
       </c>
       <c t="inlineStr" r="G24">
         <is>
-          <t xml:space="preserve">12/11/2025 16:20:00</t>
+          <t xml:space="preserve">21/11/2025 15:55:00</t>
         </is>
       </c>
       <c t="inlineStr" r="H24">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">R$ 1.00</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c t="inlineStr" r="A25">
         <is>
-          <t xml:space="preserve">Testeeeee</t>
+          <t xml:space="preserve">teste</t>
         </is>
       </c>
       <c t="inlineStr" r="B25">
         <is>
-          <t xml:space="preserve">R$ 2.00</t>
+          <t xml:space="preserve">R$ 5.00</t>
         </is>
       </c>
       <c r="C25" s="65">
-        <v>2222</v>
+        <v>123</v>
       </c>
       <c t="n" r="D25">
-        <v>100</v>
+        <v>5</v>
       </c>
       <c t="n" r="E25">
         <v>0</v>
       </c>
       <c t="inlineStr" r="F25">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">18/11/2025 13:45:00</t>
         </is>
       </c>
       <c t="inlineStr" r="G25">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">19/11/2025 14:50:00</t>
         </is>
       </c>
       <c t="inlineStr" r="H25">
@@ -1061,7 +1060,7 @@
     <row r="26">
       <c t="inlineStr" r="A26">
         <is>
-          <t xml:space="preserve">Teste17/11</t>
+          <t xml:space="preserve">testes 2111</t>
         </is>
       </c>
       <c r="B26" s="56">
@@ -1069,20 +1068,23 @@
       </c>
       <c t="inlineStr" r="C26">
         <is>
-          <t xml:space="preserve">Teste17/11</t>
-        </is>
+          <t xml:space="preserve">date123</t>
+        </is>
+      </c>
+      <c t="n" r="D26">
+        <v>5</v>
       </c>
       <c t="n" r="E26">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c t="inlineStr" r="F26">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">18/11/2025 15:55:00</t>
         </is>
       </c>
       <c t="inlineStr" r="G26">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">19/11/2025 19:55:00</t>
         </is>
       </c>
       <c t="inlineStr" r="H26">
@@ -1094,65 +1096,68 @@
     <row r="27">
       <c t="inlineStr" r="A27">
         <is>
-          <t xml:space="preserve">teste</t>
-        </is>
-      </c>
-      <c r="B27" s="56">
-        <v>0.5</v>
-      </c>
-      <c r="C27" s="65">
-        <v>5050</v>
+          <t xml:space="preserve">Teste 04/12-1</t>
+        </is>
+      </c>
+      <c t="inlineStr" r="B27">
+        <is>
+          <t xml:space="preserve">R$ 1.00</t>
+        </is>
+      </c>
+      <c t="inlineStr" r="C27">
+        <is>
+          <t xml:space="preserve">Teste 04/12-1</t>
+        </is>
       </c>
       <c t="n" r="D27">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c t="n" r="E27">
         <v>1</v>
       </c>
       <c t="inlineStr" r="F27">
         <is>
-          <t xml:space="preserve">21/11/2025 14:55:00</t>
+          <t xml:space="preserve">04/12/2025 10:45:00</t>
         </is>
       </c>
       <c t="inlineStr" r="G27">
         <is>
-          <t xml:space="preserve">21/11/2025 15:55:00</t>
+          <t xml:space="preserve">04/12/2025 10:55:00</t>
         </is>
       </c>
       <c t="inlineStr" r="H27">
         <is>
-          <t xml:space="preserve">R$ 1.00</t>
+          <t xml:space="preserve">R$ 5.00</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c t="inlineStr" r="A28">
         <is>
-          <t xml:space="preserve">teste</t>
+          <t xml:space="preserve">TesteDois</t>
         </is>
       </c>
       <c t="inlineStr" r="B28">
         <is>
-          <t xml:space="preserve">R$ 5.00</t>
-        </is>
-      </c>
-      <c r="C28" s="65">
-        <v>123</v>
-      </c>
-      <c t="n" r="D28">
-        <v>5</v>
+          <t xml:space="preserve">R$ 2.00</t>
+        </is>
+      </c>
+      <c t="inlineStr" r="C28">
+        <is>
+          <t xml:space="preserve">TesteDois</t>
+        </is>
       </c>
       <c t="n" r="E28">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c t="inlineStr" r="F28">
         <is>
-          <t xml:space="preserve">18/11/2025 13:45:00</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c t="inlineStr" r="G28">
         <is>
-          <t xml:space="preserve">19/11/2025 14:50:00</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c t="inlineStr" r="H28">
@@ -1164,7 +1169,7 @@
     <row r="29">
       <c t="inlineStr" r="A29">
         <is>
-          <t xml:space="preserve">testes 2111</t>
+          <t xml:space="preserve">CUPOM COM LIMITE 1</t>
         </is>
       </c>
       <c r="B29" s="56">
@@ -1172,23 +1177,23 @@
       </c>
       <c t="inlineStr" r="C29">
         <is>
-          <t xml:space="preserve">date123</t>
+          <t xml:space="preserve">limitado</t>
         </is>
       </c>
       <c t="n" r="D29">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c t="n" r="E29">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c t="inlineStr" r="F29">
         <is>
-          <t xml:space="preserve">18/11/2025 15:55:00</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c t="inlineStr" r="G29">
         <is>
-          <t xml:space="preserve">19/11/2025 19:55:00</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c t="inlineStr" r="H29">
@@ -1200,59 +1205,57 @@
     <row r="30">
       <c t="inlineStr" r="A30">
         <is>
-          <t xml:space="preserve">Teste 04/12-1</t>
+          <t xml:space="preserve">expirado</t>
         </is>
       </c>
       <c t="inlineStr" r="B30">
         <is>
-          <t xml:space="preserve">R$ 1.00</t>
+          <t xml:space="preserve">R$ 5.00</t>
         </is>
       </c>
       <c t="inlineStr" r="C30">
         <is>
-          <t xml:space="preserve">Teste 04/12-1</t>
-        </is>
-      </c>
-      <c t="n" r="D30">
-        <v>1</v>
+          <t xml:space="preserve">acabou50</t>
+        </is>
       </c>
       <c t="n" r="E30">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c t="inlineStr" r="F30">
         <is>
-          <t xml:space="preserve">04/12/2025 10:45:00</t>
+          <t xml:space="preserve">04/12/2025 13:00:00</t>
         </is>
       </c>
       <c t="inlineStr" r="G30">
         <is>
-          <t xml:space="preserve">04/12/2025 10:55:00</t>
+          <t xml:space="preserve">05/12/2025 09:00:00</t>
         </is>
       </c>
       <c t="inlineStr" r="H30">
         <is>
-          <t xml:space="preserve">R$ 5.00</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c t="inlineStr" r="A31">
         <is>
-          <t xml:space="preserve">TesteDois</t>
-        </is>
-      </c>
-      <c t="inlineStr" r="B31">
-        <is>
-          <t xml:space="preserve">R$ 2.00</t>
-        </is>
+          <t xml:space="preserve">cupom teste % 08/12/2025</t>
+        </is>
+      </c>
+      <c r="B31" s="56">
+        <v>0.5</v>
       </c>
       <c t="inlineStr" r="C31">
         <is>
-          <t xml:space="preserve">TesteDois</t>
-        </is>
+          <t xml:space="preserve">08122025</t>
+        </is>
+      </c>
+      <c t="n" r="D31">
+        <v>1</v>
       </c>
       <c t="n" r="E31">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c t="inlineStr" r="F31">
         <is>
@@ -1273,31 +1276,30 @@
     <row r="32">
       <c t="inlineStr" r="A32">
         <is>
-          <t xml:space="preserve">CUPOM COM LIMITE 1</t>
-        </is>
-      </c>
-      <c r="B32" s="56">
-        <v>0.5</v>
+          <t xml:space="preserve">cupom data expirada 08/12/2025</t>
+        </is>
+      </c>
+      <c t="inlineStr" r="B32">
+        <is>
+          <t xml:space="preserve">R$ 5.00</t>
+        </is>
       </c>
       <c t="inlineStr" r="C32">
         <is>
-          <t xml:space="preserve">limitado</t>
-        </is>
-      </c>
-      <c t="n" r="D32">
-        <v>1</v>
+          <t xml:space="preserve">0802200511</t>
+        </is>
       </c>
       <c t="n" r="E32">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c t="inlineStr" r="F32">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">01/12/2025 04:00:00</t>
         </is>
       </c>
       <c t="inlineStr" r="G32">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">02/12/2025 01:05:00</t>
         </is>
       </c>
       <c t="inlineStr" r="H32">
@@ -1309,30 +1311,31 @@
     <row r="33">
       <c t="inlineStr" r="A33">
         <is>
-          <t xml:space="preserve">expirado</t>
-        </is>
-      </c>
-      <c t="inlineStr" r="B33">
-        <is>
-          <t xml:space="preserve">R$ 5.00</t>
-        </is>
+          <t xml:space="preserve">Teste</t>
+        </is>
+      </c>
+      <c r="B33" s="56">
+        <v>0.5</v>
       </c>
       <c t="inlineStr" r="C33">
         <is>
-          <t xml:space="preserve">acabou50</t>
-        </is>
+          <t xml:space="preserve">0912</t>
+        </is>
+      </c>
+      <c t="n" r="D33">
+        <v>1</v>
       </c>
       <c t="n" r="E33">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c t="inlineStr" r="F33">
         <is>
-          <t xml:space="preserve">04/12/2025 13:00:00</t>
+          <t xml:space="preserve">09/12/2025 11:00:00</t>
         </is>
       </c>
       <c t="inlineStr" r="G33">
         <is>
-          <t xml:space="preserve">05/12/2025 09:00:00</t>
+          <t xml:space="preserve">09/12/2025 15:00:00</t>
         </is>
       </c>
       <c t="inlineStr" r="H33">
@@ -1344,15 +1347,17 @@
     <row r="34">
       <c t="inlineStr" r="A34">
         <is>
-          <t xml:space="preserve">cupom teste % 08/12/2025</t>
-        </is>
-      </c>
-      <c r="B34" s="56">
-        <v>0.5</v>
+          <t xml:space="preserve">Teste Teste</t>
+        </is>
+      </c>
+      <c t="inlineStr" r="B34">
+        <is>
+          <t xml:space="preserve">R$ 1.00</t>
+        </is>
       </c>
       <c t="inlineStr" r="C34">
         <is>
-          <t xml:space="preserve">08122025</t>
+          <t xml:space="preserve">09121</t>
         </is>
       </c>
       <c t="n" r="D34">
@@ -1380,17 +1385,17 @@
     <row r="35">
       <c t="inlineStr" r="A35">
         <is>
-          <t xml:space="preserve">cupom data expirada 08/12/2025</t>
+          <t xml:space="preserve">Teste 2</t>
         </is>
       </c>
       <c t="inlineStr" r="B35">
         <is>
-          <t xml:space="preserve">R$ 5.00</t>
+          <t xml:space="preserve">R$ 1.00</t>
         </is>
       </c>
       <c t="inlineStr" r="C35">
         <is>
-          <t xml:space="preserve">0802200511</t>
+          <t xml:space="preserve">09122</t>
         </is>
       </c>
       <c t="n" r="E35">
@@ -1398,12 +1403,12 @@
       </c>
       <c t="inlineStr" r="F35">
         <is>
-          <t xml:space="preserve">01/12/2025 04:00:00</t>
+          <t xml:space="preserve">09/12/2025 12:00:00</t>
         </is>
       </c>
       <c t="inlineStr" r="G35">
         <is>
-          <t xml:space="preserve">02/12/2025 01:05:00</t>
+          <t xml:space="preserve">09/12/2025 13:10:00</t>
         </is>
       </c>
       <c t="inlineStr" r="H35">
@@ -1415,15 +1420,15 @@
     <row r="36">
       <c t="inlineStr" r="A36">
         <is>
-          <t xml:space="preserve">Teste</t>
+          <t xml:space="preserve">cupom 09/12/25</t>
         </is>
       </c>
       <c r="B36" s="56">
-        <v>0.5</v>
+        <v>0.11</v>
       </c>
       <c t="inlineStr" r="C36">
         <is>
-          <t xml:space="preserve">0912</t>
+          <t xml:space="preserve">cupom101010</t>
         </is>
       </c>
       <c t="n" r="D36">
@@ -1439,45 +1444,45 @@
       </c>
       <c t="inlineStr" r="G36">
         <is>
-          <t xml:space="preserve">09/12/2025 15:00:00</t>
+          <t xml:space="preserve">09/12/2025 19:55:00</t>
         </is>
       </c>
       <c t="inlineStr" r="H36">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">R$ 2.00</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c t="inlineStr" r="A37">
         <is>
-          <t xml:space="preserve">Teste Teste</t>
+          <t xml:space="preserve">cupom29929</t>
         </is>
       </c>
       <c t="inlineStr" r="B37">
         <is>
-          <t xml:space="preserve">R$ 1.00</t>
+          <t xml:space="preserve">R$ 5.00</t>
         </is>
       </c>
       <c t="inlineStr" r="C37">
         <is>
-          <t xml:space="preserve">09121</t>
+          <t xml:space="preserve">09082025</t>
         </is>
       </c>
       <c t="n" r="D37">
         <v>1</v>
       </c>
       <c t="n" r="E37">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c t="inlineStr" r="F37">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">09/12/2025 09:00:00</t>
         </is>
       </c>
       <c t="inlineStr" r="G37">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">09/12/2025 10:00:00</t>
         </is>
       </c>
       <c t="inlineStr" r="H37">
@@ -1489,30 +1494,31 @@
     <row r="38">
       <c t="inlineStr" r="A38">
         <is>
-          <t xml:space="preserve">Teste 2</t>
+          <t xml:space="preserve">cupom data encerradda</t>
         </is>
       </c>
       <c t="inlineStr" r="B38">
         <is>
-          <t xml:space="preserve">R$ 1.00</t>
-        </is>
-      </c>
-      <c t="inlineStr" r="C38">
-        <is>
-          <t xml:space="preserve">09122</t>
-        </is>
+          <t xml:space="preserve">R$ 5.00</t>
+        </is>
+      </c>
+      <c r="C38" s="65">
+        <v>898989</v>
+      </c>
+      <c t="n" r="D38">
+        <v>2</v>
       </c>
       <c t="n" r="E38">
         <v>0</v>
       </c>
       <c t="inlineStr" r="F38">
         <is>
-          <t xml:space="preserve">09/12/2025 12:00:00</t>
+          <t xml:space="preserve">01/11/2025 02:10:00</t>
         </is>
       </c>
       <c t="inlineStr" r="G38">
         <is>
-          <t xml:space="preserve">09/12/2025 13:10:00</t>
+          <t xml:space="preserve">02/12/2025 01:05:00</t>
         </is>
       </c>
       <c t="inlineStr" r="H38">
@@ -1524,69 +1530,66 @@
     <row r="39">
       <c t="inlineStr" r="A39">
         <is>
-          <t xml:space="preserve">cupom 09/12/25</t>
+          <t xml:space="preserve">turma recorrente</t>
         </is>
       </c>
       <c r="B39" s="56">
-        <v>0.11</v>
+        <v>0.1</v>
       </c>
       <c t="inlineStr" r="C39">
         <is>
-          <t xml:space="preserve">cupom101010</t>
-        </is>
-      </c>
-      <c t="n" r="D39">
-        <v>1</v>
+          <t xml:space="preserve">teste09122025</t>
+        </is>
       </c>
       <c t="n" r="E39">
         <v>1</v>
       </c>
       <c t="inlineStr" r="F39">
         <is>
-          <t xml:space="preserve">09/12/2025 11:00:00</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c t="inlineStr" r="G39">
         <is>
-          <t xml:space="preserve">09/12/2025 19:55:00</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c t="inlineStr" r="H39">
         <is>
-          <t xml:space="preserve">R$ 2.00</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c t="inlineStr" r="A40">
         <is>
-          <t xml:space="preserve">cupom29929</t>
+          <t xml:space="preserve">Teste 12/12-2</t>
         </is>
       </c>
       <c t="inlineStr" r="B40">
         <is>
-          <t xml:space="preserve">R$ 5.00</t>
+          <t xml:space="preserve">R$ 1.00</t>
         </is>
       </c>
       <c t="inlineStr" r="C40">
         <is>
-          <t xml:space="preserve">09082025</t>
+          <t xml:space="preserve">Teste 12/12-2</t>
         </is>
       </c>
       <c t="n" r="D40">
         <v>1</v>
       </c>
       <c t="n" r="E40">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c t="inlineStr" r="F40">
         <is>
-          <t xml:space="preserve">09/12/2025 09:00:00</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c t="inlineStr" r="G40">
         <is>
-          <t xml:space="preserve">09/12/2025 10:00:00</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c t="inlineStr" r="H40">
@@ -1598,7 +1601,7 @@
     <row r="41">
       <c t="inlineStr" r="A41">
         <is>
-          <t xml:space="preserve">cupom data encerradda</t>
+          <t xml:space="preserve">caio expiração teste</t>
         </is>
       </c>
       <c t="inlineStr" r="B41">
@@ -1606,23 +1609,25 @@
           <t xml:space="preserve">R$ 5.00</t>
         </is>
       </c>
-      <c r="C41" s="65">
-        <v>898989</v>
+      <c t="inlineStr" r="C41">
+        <is>
+          <t xml:space="preserve">caiocaiocaio</t>
+        </is>
       </c>
       <c t="n" r="D41">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c t="n" r="E41">
         <v>0</v>
       </c>
       <c t="inlineStr" r="F41">
         <is>
-          <t xml:space="preserve">01/11/2025 02:10:00</t>
+          <t xml:space="preserve">12/12/2025 11:00:00</t>
         </is>
       </c>
       <c t="inlineStr" r="G41">
         <is>
-          <t xml:space="preserve">02/12/2025 01:05:00</t>
+          <t xml:space="preserve">12/12/2025 11:30:00</t>
         </is>
       </c>
       <c t="inlineStr" r="H41">
@@ -1634,19 +1639,24 @@
     <row r="42">
       <c t="inlineStr" r="A42">
         <is>
-          <t xml:space="preserve">turma recorrente</t>
-        </is>
-      </c>
-      <c r="B42" s="56">
-        <v>0.1</v>
+          <t xml:space="preserve">teste limite</t>
+        </is>
+      </c>
+      <c t="inlineStr" r="B42">
+        <is>
+          <t xml:space="preserve">R$ 1.00</t>
+        </is>
       </c>
       <c t="inlineStr" r="C42">
         <is>
-          <t xml:space="preserve">teste09122025</t>
-        </is>
+          <t xml:space="preserve">testelimitete</t>
+        </is>
+      </c>
+      <c t="n" r="D42">
+        <v>1</v>
       </c>
       <c t="n" r="E42">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c t="inlineStr" r="F42">
         <is>
@@ -1660,40 +1670,38 @@
       </c>
       <c t="inlineStr" r="H42">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">R$ 5.00</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c t="inlineStr" r="A43">
         <is>
-          <t xml:space="preserve">Teste 12/12-2</t>
-        </is>
-      </c>
-      <c t="inlineStr" r="B43">
-        <is>
-          <t xml:space="preserve">R$ 1.00</t>
-        </is>
+          <t xml:space="preserve">12/12 - 2</t>
+        </is>
+      </c>
+      <c r="B43" s="56">
+        <v>0.5</v>
       </c>
       <c t="inlineStr" r="C43">
         <is>
-          <t xml:space="preserve">Teste 12/12-2</t>
+          <t xml:space="preserve">12/12 - 2</t>
         </is>
       </c>
       <c t="n" r="D43">
         <v>1</v>
       </c>
       <c t="n" r="E43">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c t="inlineStr" r="F43">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">12/12/2025 00:00:00</t>
         </is>
       </c>
       <c t="inlineStr" r="G43">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">12/12/2025 23:55:00</t>
         </is>
       </c>
       <c t="inlineStr" r="H43">
@@ -1705,33 +1713,31 @@
     <row r="44">
       <c t="inlineStr" r="A44">
         <is>
-          <t xml:space="preserve">caio expiração teste</t>
-        </is>
-      </c>
-      <c t="inlineStr" r="B44">
-        <is>
-          <t xml:space="preserve">R$ 5.00</t>
-        </is>
+          <t xml:space="preserve">18/12</t>
+        </is>
+      </c>
+      <c r="B44" s="56">
+        <v>0.5</v>
       </c>
       <c t="inlineStr" r="C44">
         <is>
-          <t xml:space="preserve">caiocaiocaio</t>
+          <t xml:space="preserve">18/12</t>
         </is>
       </c>
       <c t="n" r="D44">
-        <v>5</v>
+        <v>99</v>
       </c>
       <c t="n" r="E44">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c t="inlineStr" r="F44">
         <is>
-          <t xml:space="preserve">12/12/2025 11:00:00</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c t="inlineStr" r="G44">
         <is>
-          <t xml:space="preserve">12/12/2025 11:30:00</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c t="inlineStr" r="H44">
@@ -1743,24 +1749,22 @@
     <row r="45">
       <c t="inlineStr" r="A45">
         <is>
-          <t xml:space="preserve">teste limite</t>
-        </is>
-      </c>
-      <c t="inlineStr" r="B45">
-        <is>
-          <t xml:space="preserve">R$ 1.00</t>
-        </is>
+          <t xml:space="preserve">Trila chefcklist 18/12/25</t>
+        </is>
+      </c>
+      <c r="B45" s="56">
+        <v>0.5</v>
       </c>
       <c t="inlineStr" r="C45">
         <is>
-          <t xml:space="preserve">testelimitete</t>
+          <t xml:space="preserve">caio18122025</t>
         </is>
       </c>
       <c t="n" r="D45">
         <v>1</v>
       </c>
       <c t="n" r="E45">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c t="inlineStr" r="F45">
         <is>
@@ -1774,38 +1778,34 @@
       </c>
       <c t="inlineStr" r="H45">
         <is>
-          <t xml:space="preserve">R$ 5.00</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
     </row>
     <row r="46">
-      <c t="inlineStr" r="A46">
-        <is>
-          <t xml:space="preserve">12/12 - 2</t>
-        </is>
+      <c r="A46" s="56">
+        <v>1</v>
       </c>
       <c r="B46" s="56">
-        <v>0.5</v>
-      </c>
-      <c t="inlineStr" r="C46">
-        <is>
-          <t xml:space="preserve">12/12 - 2</t>
-        </is>
+        <v>1</v>
+      </c>
+      <c r="C46" s="56">
+        <v>1</v>
       </c>
       <c t="n" r="D46">
-        <v>1</v>
+        <v>99</v>
       </c>
       <c t="n" r="E46">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c t="inlineStr" r="F46">
         <is>
-          <t xml:space="preserve">12/12/2025 00:00:00</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c t="inlineStr" r="G46">
         <is>
-          <t xml:space="preserve">12/12/2025 23:55:00</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c t="inlineStr" r="H46">
@@ -1817,22 +1817,21 @@
     <row r="47">
       <c t="inlineStr" r="A47">
         <is>
-          <t xml:space="preserve">18/12</t>
-        </is>
-      </c>
-      <c r="B47" s="56">
-        <v>0.5</v>
+          <t xml:space="preserve">18/12  cupom</t>
+        </is>
+      </c>
+      <c t="inlineStr" r="B47">
+        <is>
+          <t xml:space="preserve">R$ 10.00</t>
+        </is>
       </c>
       <c t="inlineStr" r="C47">
         <is>
-          <t xml:space="preserve">18/12</t>
-        </is>
-      </c>
-      <c t="n" r="D47">
-        <v>99</v>
+          <t xml:space="preserve">18/12cupom</t>
+        </is>
       </c>
       <c t="n" r="E47">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c t="inlineStr" r="F47">
         <is>
@@ -1853,7 +1852,7 @@
     <row r="48">
       <c t="inlineStr" r="A48">
         <is>
-          <t xml:space="preserve">Trila chefcklist 18/12/25</t>
+          <t xml:space="preserve">cupom 50%</t>
         </is>
       </c>
       <c r="B48" s="56">
@@ -1861,14 +1860,14 @@
       </c>
       <c t="inlineStr" r="C48">
         <is>
-          <t xml:space="preserve">caio18122025</t>
+          <t xml:space="preserve">50%1812</t>
         </is>
       </c>
       <c t="n" r="D48">
         <v>1</v>
       </c>
       <c t="n" r="E48">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c t="inlineStr" r="F48">
         <is>
@@ -1887,20 +1886,21 @@
       </c>
     </row>
     <row r="49">
-      <c r="A49" s="56">
-        <v>1</v>
-      </c>
-      <c r="B49" s="56">
-        <v>1</v>
-      </c>
-      <c r="C49" s="56">
-        <v>1</v>
-      </c>
-      <c t="n" r="D49">
-        <v>99</v>
+      <c t="inlineStr" r="A49">
+        <is>
+          <t xml:space="preserve">teste</t>
+        </is>
+      </c>
+      <c t="inlineStr" r="B49">
+        <is>
+          <t xml:space="preserve">R$ 1.00</t>
+        </is>
+      </c>
+      <c r="C49" s="65">
+        <v>969754</v>
       </c>
       <c t="n" r="E49">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c t="inlineStr" r="F49">
         <is>
@@ -1914,28 +1914,26 @@
       </c>
       <c t="inlineStr" r="H49">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">R$ 1.00</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c t="inlineStr" r="A50">
         <is>
-          <t xml:space="preserve">18/12  cupom</t>
-        </is>
-      </c>
-      <c t="inlineStr" r="B50">
-        <is>
-          <t xml:space="preserve">R$ 10.00</t>
-        </is>
+          <t xml:space="preserve">teste metade</t>
+        </is>
+      </c>
+      <c r="B50" s="56">
+        <v>0.5</v>
       </c>
       <c t="inlineStr" r="C50">
         <is>
-          <t xml:space="preserve">18/12cupom</t>
+          <t xml:space="preserve">0510</t>
         </is>
       </c>
       <c t="n" r="E50">
-        <v>1</v>
+        <v>18</v>
       </c>
       <c t="inlineStr" r="F50">
         <is>
@@ -1956,7 +1954,7 @@
     <row r="51">
       <c t="inlineStr" r="A51">
         <is>
-          <t xml:space="preserve">cupom 50%</t>
+          <t xml:space="preserve">TesteLimite</t>
         </is>
       </c>
       <c r="B51" s="56">
@@ -1964,14 +1962,14 @@
       </c>
       <c t="inlineStr" r="C51">
         <is>
-          <t xml:space="preserve">50%1812</t>
+          <t xml:space="preserve">05/01/2026</t>
         </is>
       </c>
       <c t="n" r="D51">
         <v>1</v>
       </c>
       <c t="n" r="E51">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c t="inlineStr" r="F51">
         <is>
@@ -1992,52 +1990,54 @@
     <row r="52">
       <c t="inlineStr" r="A52">
         <is>
-          <t xml:space="preserve">teste</t>
-        </is>
-      </c>
-      <c t="inlineStr" r="B52">
-        <is>
-          <t xml:space="preserve">R$ 1.00</t>
-        </is>
-      </c>
-      <c r="C52" s="65">
-        <v>969754</v>
+          <t xml:space="preserve">Data expirada</t>
+        </is>
+      </c>
+      <c r="B52" s="56">
+        <v>0.5</v>
+      </c>
+      <c t="inlineStr" r="C52">
+        <is>
+          <t xml:space="preserve">0520</t>
+        </is>
       </c>
       <c t="n" r="E52">
         <v>0</v>
       </c>
       <c t="inlineStr" r="F52">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">05/01/2026 14:00:00</t>
         </is>
       </c>
       <c t="inlineStr" r="G52">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">05/01/2026 14:15:00</t>
         </is>
       </c>
       <c t="inlineStr" r="H52">
         <is>
-          <t xml:space="preserve">R$ 1.00</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c t="inlineStr" r="A53">
         <is>
-          <t xml:space="preserve">teste metade</t>
-        </is>
-      </c>
-      <c r="B53" s="56">
-        <v>0.5</v>
+          <t xml:space="preserve">Valor Acima do minimo</t>
+        </is>
+      </c>
+      <c t="inlineStr" r="B53">
+        <is>
+          <t xml:space="preserve">R$ 1.00</t>
+        </is>
       </c>
       <c t="inlineStr" r="C53">
         <is>
-          <t xml:space="preserve">0510</t>
+          <t xml:space="preserve">0530</t>
         </is>
       </c>
       <c t="n" r="E53">
-        <v>18</v>
+        <v>1</v>
       </c>
       <c t="inlineStr" r="F53">
         <is>
@@ -2051,38 +2051,40 @@
       </c>
       <c t="inlineStr" r="H53">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">R$ 2.00</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c t="inlineStr" r="A54">
         <is>
-          <t xml:space="preserve">TesteLimite</t>
-        </is>
-      </c>
-      <c r="B54" s="56">
-        <v>0.5</v>
+          <t xml:space="preserve">teste cupom recorrente</t>
+        </is>
+      </c>
+      <c t="inlineStr" r="B54">
+        <is>
+          <t xml:space="preserve">R$ 5.00</t>
+        </is>
       </c>
       <c t="inlineStr" r="C54">
         <is>
-          <t xml:space="preserve">05/01/2026</t>
+          <t xml:space="preserve">cinco reais</t>
         </is>
       </c>
       <c t="n" r="D54">
         <v>1</v>
       </c>
       <c t="n" r="E54">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c t="inlineStr" r="F54">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">06/01/2026 15:00:00</t>
         </is>
       </c>
       <c t="inlineStr" r="G54">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">06/01/2026 16:05:00</t>
         </is>
       </c>
       <c t="inlineStr" r="H54">
@@ -2094,28 +2096,31 @@
     <row r="55">
       <c t="inlineStr" r="A55">
         <is>
-          <t xml:space="preserve">Data expirada</t>
+          <t xml:space="preserve">teste06/01</t>
         </is>
       </c>
       <c r="B55" s="56">
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c t="inlineStr" r="C55">
         <is>
-          <t xml:space="preserve">0520</t>
-        </is>
+          <t xml:space="preserve">teste06/01</t>
+        </is>
+      </c>
+      <c t="n" r="D55">
+        <v>100</v>
       </c>
       <c t="n" r="E55">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c t="inlineStr" r="F55">
         <is>
-          <t xml:space="preserve">05/01/2026 14:00:00</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c t="inlineStr" r="G55">
         <is>
-          <t xml:space="preserve">05/01/2026 14:15:00</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c t="inlineStr" r="H55">
@@ -2127,7 +2132,7 @@
     <row r="56">
       <c t="inlineStr" r="A56">
         <is>
-          <t xml:space="preserve">Valor Acima do minimo</t>
+          <t xml:space="preserve">teste</t>
         </is>
       </c>
       <c t="inlineStr" r="B56">
@@ -2135,10 +2140,11 @@
           <t xml:space="preserve">R$ 1.00</t>
         </is>
       </c>
-      <c t="inlineStr" r="C56">
-        <is>
-          <t xml:space="preserve">0530</t>
-        </is>
+      <c r="C56" s="65">
+        <v>1301</v>
+      </c>
+      <c t="n" r="D56">
+        <v>1</v>
       </c>
       <c t="n" r="E56">
         <v>1</v>
@@ -2155,40 +2161,33 @@
       </c>
       <c t="inlineStr" r="H56">
         <is>
-          <t xml:space="preserve">R$ 2.00</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c t="inlineStr" r="A57">
         <is>
-          <t xml:space="preserve">teste cupom recorrente</t>
-        </is>
-      </c>
-      <c t="inlineStr" r="B57">
-        <is>
-          <t xml:space="preserve">R$ 5.00</t>
-        </is>
-      </c>
-      <c t="inlineStr" r="C57">
-        <is>
-          <t xml:space="preserve">cinco reais</t>
-        </is>
-      </c>
-      <c t="n" r="D57">
-        <v>1</v>
+          <t xml:space="preserve">teste2</t>
+        </is>
+      </c>
+      <c r="B57" s="56">
+        <v>0.5</v>
+      </c>
+      <c r="C57" s="65">
+        <v>1302</v>
       </c>
       <c t="n" r="E57">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c t="inlineStr" r="F57">
         <is>
-          <t xml:space="preserve">06/01/2026 15:00:00</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c t="inlineStr" r="G57">
         <is>
-          <t xml:space="preserve">06/01/2026 16:05:00</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c t="inlineStr" r="H57">
@@ -2200,22 +2199,21 @@
     <row r="58">
       <c t="inlineStr" r="A58">
         <is>
-          <t xml:space="preserve">teste06/01</t>
-        </is>
-      </c>
-      <c r="B58" s="56">
-        <v>1</v>
+          <t xml:space="preserve">Desconto1</t>
+        </is>
+      </c>
+      <c t="inlineStr" r="B58">
+        <is>
+          <t xml:space="preserve">R$ 1.00</t>
+        </is>
       </c>
       <c t="inlineStr" r="C58">
         <is>
-          <t xml:space="preserve">teste06/01</t>
-        </is>
-      </c>
-      <c t="n" r="D58">
-        <v>100</v>
+          <t xml:space="preserve">desc1</t>
+        </is>
       </c>
       <c t="n" r="E58">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c t="inlineStr" r="F58">
         <is>
@@ -2236,22 +2234,24 @@
     <row r="59">
       <c t="inlineStr" r="A59">
         <is>
-          <t xml:space="preserve">teste</t>
+          <t xml:space="preserve">Desconto2</t>
         </is>
       </c>
       <c t="inlineStr" r="B59">
         <is>
-          <t xml:space="preserve">R$ 1.00</t>
-        </is>
-      </c>
-      <c r="C59" s="65">
-        <v>1301</v>
+          <t xml:space="preserve">R$ 2.00</t>
+        </is>
+      </c>
+      <c t="inlineStr" r="C59">
+        <is>
+          <t xml:space="preserve">desc2</t>
+        </is>
       </c>
       <c t="n" r="D59">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c t="n" r="E59">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c t="inlineStr" r="F59">
         <is>
@@ -2272,14 +2272,17 @@
     <row r="60">
       <c t="inlineStr" r="A60">
         <is>
-          <t xml:space="preserve">teste2</t>
+          <t xml:space="preserve">TesteLector14</t>
         </is>
       </c>
       <c r="B60" s="56">
         <v>0.5</v>
       </c>
       <c r="C60" s="65">
-        <v>1302</v>
+        <v>12345678</v>
+      </c>
+      <c t="n" r="D60">
+        <v>1</v>
       </c>
       <c t="n" r="E60">
         <v>1</v>
@@ -2303,7 +2306,7 @@
     <row r="61">
       <c t="inlineStr" r="A61">
         <is>
-          <t xml:space="preserve">Desconto1</t>
+          <t xml:space="preserve">Teste141414</t>
         </is>
       </c>
       <c t="inlineStr" r="B61">
@@ -2311,13 +2314,14 @@
           <t xml:space="preserve">R$ 1.00</t>
         </is>
       </c>
-      <c t="inlineStr" r="C61">
-        <is>
-          <t xml:space="preserve">desc1</t>
-        </is>
+      <c r="C61" s="65">
+        <v>123456789</v>
+      </c>
+      <c t="n" r="D61">
+        <v>1</v>
       </c>
       <c t="n" r="E61">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c t="inlineStr" r="F61">
         <is>
@@ -2338,21 +2342,16 @@
     <row r="62">
       <c t="inlineStr" r="A62">
         <is>
-          <t xml:space="preserve">Desconto2</t>
-        </is>
-      </c>
-      <c t="inlineStr" r="B62">
-        <is>
-          <t xml:space="preserve">R$ 2.00</t>
-        </is>
+          <t xml:space="preserve">15/01</t>
+        </is>
+      </c>
+      <c r="B62" s="56">
+        <v>0.5</v>
       </c>
       <c t="inlineStr" r="C62">
         <is>
-          <t xml:space="preserve">desc2</t>
-        </is>
-      </c>
-      <c t="n" r="D62">
-        <v>10</v>
+          <t xml:space="preserve">15/01</t>
+        </is>
       </c>
       <c t="n" r="E62">
         <v>0</v>
@@ -2376,14 +2375,16 @@
     <row r="63">
       <c t="inlineStr" r="A63">
         <is>
-          <t xml:space="preserve">TesteLector14</t>
+          <t xml:space="preserve">15/01</t>
         </is>
       </c>
       <c r="B63" s="56">
-        <v>0.5</v>
-      </c>
-      <c r="C63" s="65">
-        <v>12345678</v>
+        <v>1</v>
+      </c>
+      <c t="inlineStr" r="C63">
+        <is>
+          <t xml:space="preserve">15/01%</t>
+        </is>
       </c>
       <c t="n" r="D63">
         <v>1</v>
@@ -2393,12 +2394,12 @@
       </c>
       <c t="inlineStr" r="F63">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">15/01/2026 12:00:00</t>
         </is>
       </c>
       <c t="inlineStr" r="G63">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">15/01/2026 14:00:00</t>
         </is>
       </c>
       <c t="inlineStr" r="H63">
@@ -2410,16 +2411,14 @@
     <row r="64">
       <c t="inlineStr" r="A64">
         <is>
-          <t xml:space="preserve">Teste141414</t>
-        </is>
-      </c>
-      <c t="inlineStr" r="B64">
-        <is>
-          <t xml:space="preserve">R$ 1.00</t>
-        </is>
+          <t xml:space="preserve">Teste 1515</t>
+        </is>
+      </c>
+      <c r="B64" s="56">
+        <v>0.3</v>
       </c>
       <c r="C64" s="65">
-        <v>123456789</v>
+        <v>1515</v>
       </c>
       <c t="n" r="D64">
         <v>1</v>
@@ -2446,28 +2445,28 @@
     <row r="65">
       <c t="inlineStr" r="A65">
         <is>
-          <t xml:space="preserve">15/01</t>
-        </is>
-      </c>
-      <c r="B65" s="56">
-        <v>0.5</v>
-      </c>
-      <c t="inlineStr" r="C65">
-        <is>
-          <t xml:space="preserve">15/01</t>
-        </is>
+          <t xml:space="preserve">Teste 151515</t>
+        </is>
+      </c>
+      <c t="inlineStr" r="B65">
+        <is>
+          <t xml:space="preserve">R$ 1.00</t>
+        </is>
+      </c>
+      <c r="C65" s="65">
+        <v>151515</v>
       </c>
       <c t="n" r="E65">
         <v>0</v>
       </c>
       <c t="inlineStr" r="F65">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">15/01/2026 14:05:00</t>
         </is>
       </c>
       <c t="inlineStr" r="G65">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">15/01/2026 14:05:00</t>
         </is>
       </c>
       <c t="inlineStr" r="H65">
@@ -2479,31 +2478,28 @@
     <row r="66">
       <c t="inlineStr" r="A66">
         <is>
-          <t xml:space="preserve">15/01</t>
-        </is>
-      </c>
-      <c r="B66" s="56">
-        <v>1</v>
-      </c>
-      <c t="inlineStr" r="C66">
-        <is>
-          <t xml:space="preserve">15/01%</t>
-        </is>
-      </c>
-      <c t="n" r="D66">
-        <v>1</v>
+          <t xml:space="preserve">Teste 0115</t>
+        </is>
+      </c>
+      <c t="inlineStr" r="B66">
+        <is>
+          <t xml:space="preserve">R$ 1.00</t>
+        </is>
+      </c>
+      <c r="C66" s="65">
+        <v>15151515</v>
       </c>
       <c t="n" r="E66">
         <v>1</v>
       </c>
       <c t="inlineStr" r="F66">
         <is>
-          <t xml:space="preserve">15/01/2026 12:00:00</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c t="inlineStr" r="G66">
         <is>
-          <t xml:space="preserve">15/01/2026 14:00:00</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c t="inlineStr" r="H66">
@@ -2515,29 +2511,31 @@
     <row r="67">
       <c t="inlineStr" r="A67">
         <is>
-          <t xml:space="preserve">Teste 1515</t>
+          <t xml:space="preserve">teste cupom 20/01</t>
         </is>
       </c>
       <c r="B67" s="56">
         <v>0.3</v>
       </c>
-      <c r="C67" s="65">
-        <v>1515</v>
+      <c t="inlineStr" r="C67">
+        <is>
+          <t xml:space="preserve">lc202601</t>
+        </is>
       </c>
       <c t="n" r="D67">
-        <v>1</v>
+        <v>20</v>
       </c>
       <c t="n" r="E67">
         <v>1</v>
       </c>
       <c t="inlineStr" r="F67">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">20/01/2026 12:40:00</t>
         </is>
       </c>
       <c t="inlineStr" r="G67">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">29/01/2026 18:50:00</t>
         </is>
       </c>
       <c t="inlineStr" r="H67">
@@ -2549,28 +2547,29 @@
     <row r="68">
       <c t="inlineStr" r="A68">
         <is>
-          <t xml:space="preserve">Teste 151515</t>
-        </is>
-      </c>
-      <c t="inlineStr" r="B68">
-        <is>
-          <t xml:space="preserve">R$ 1.00</t>
-        </is>
+          <t xml:space="preserve">Teste 2101</t>
+        </is>
+      </c>
+      <c r="B68" s="56">
+        <v>0.5</v>
       </c>
       <c r="C68" s="65">
-        <v>151515</v>
+        <v>2101</v>
+      </c>
+      <c t="n" r="D68">
+        <v>1</v>
       </c>
       <c t="n" r="E68">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c t="inlineStr" r="F68">
         <is>
-          <t xml:space="preserve">15/01/2026 14:05:00</t>
+          <t xml:space="preserve">21/01/2026 10:55:00</t>
         </is>
       </c>
       <c t="inlineStr" r="G68">
         <is>
-          <t xml:space="preserve">15/01/2026 14:05:00</t>
+          <t xml:space="preserve">21/01/2026 11:35:00</t>
         </is>
       </c>
       <c t="inlineStr" r="H68">
@@ -2582,7 +2581,7 @@
     <row r="69">
       <c t="inlineStr" r="A69">
         <is>
-          <t xml:space="preserve">Teste 0115</t>
+          <t xml:space="preserve">Teste 2</t>
         </is>
       </c>
       <c t="inlineStr" r="B69">
@@ -2591,7 +2590,10 @@
         </is>
       </c>
       <c r="C69" s="65">
-        <v>15151515</v>
+        <v>21012</v>
+      </c>
+      <c t="n" r="D69">
+        <v>1</v>
       </c>
       <c t="n" r="E69">
         <v>1</v>
@@ -2608,38 +2610,35 @@
       </c>
       <c t="inlineStr" r="H69">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">R$ 1.00</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c t="inlineStr" r="A70">
         <is>
-          <t xml:space="preserve">teste cupom 20/01</t>
-        </is>
-      </c>
-      <c r="B70" s="56">
-        <v>0.3</v>
-      </c>
-      <c t="inlineStr" r="C70">
-        <is>
-          <t xml:space="preserve">lc202601</t>
-        </is>
-      </c>
-      <c t="n" r="D70">
-        <v>20</v>
+          <t xml:space="preserve">Teste 100% 2101</t>
+        </is>
+      </c>
+      <c t="inlineStr" r="B70">
+        <is>
+          <t xml:space="preserve">R$ 1.00</t>
+        </is>
+      </c>
+      <c r="C70" s="65">
+        <v>2006</v>
       </c>
       <c t="n" r="E70">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c t="inlineStr" r="F70">
         <is>
-          <t xml:space="preserve">20/01/2026 12:40:00</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c t="inlineStr" r="G70">
         <is>
-          <t xml:space="preserve">29/01/2026 18:50:00</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c t="inlineStr" r="H70">
@@ -2651,29 +2650,26 @@
     <row r="71">
       <c t="inlineStr" r="A71">
         <is>
-          <t xml:space="preserve">Teste 2101</t>
+          <t xml:space="preserve">Teste 21013</t>
         </is>
       </c>
       <c r="B71" s="56">
         <v>0.5</v>
       </c>
       <c r="C71" s="65">
-        <v>2101</v>
-      </c>
-      <c t="n" r="D71">
-        <v>1</v>
+        <v>21013</v>
       </c>
       <c t="n" r="E71">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c t="inlineStr" r="F71">
         <is>
-          <t xml:space="preserve">21/01/2026 10:55:00</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c t="inlineStr" r="G71">
         <is>
-          <t xml:space="preserve">21/01/2026 11:35:00</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c t="inlineStr" r="H71">
@@ -2685,55 +2681,58 @@
     <row r="72">
       <c t="inlineStr" r="A72">
         <is>
-          <t xml:space="preserve">Teste 2</t>
-        </is>
-      </c>
-      <c t="inlineStr" r="B72">
-        <is>
-          <t xml:space="preserve">R$ 1.00</t>
-        </is>
-      </c>
-      <c r="C72" s="65">
-        <v>21012</v>
+          <t xml:space="preserve">cupom teste 21/01</t>
+        </is>
+      </c>
+      <c r="B72" s="56">
+        <v>0.3</v>
+      </c>
+      <c t="inlineStr" r="C72">
+        <is>
+          <t xml:space="preserve">my20261</t>
+        </is>
       </c>
       <c t="n" r="D72">
-        <v>1</v>
+        <v>11</v>
       </c>
       <c t="n" r="E72">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c t="inlineStr" r="F72">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">21/01/2026 13:00:00</t>
         </is>
       </c>
       <c t="inlineStr" r="G72">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">21/01/2026 13:25:00</t>
         </is>
       </c>
       <c t="inlineStr" r="H72">
         <is>
-          <t xml:space="preserve">R$ 1.00</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c t="inlineStr" r="A73">
         <is>
-          <t xml:space="preserve">Teste 100% 2101</t>
-        </is>
-      </c>
-      <c t="inlineStr" r="B73">
-        <is>
-          <t xml:space="preserve">R$ 1.00</t>
-        </is>
-      </c>
-      <c r="C73" s="65">
-        <v>2006</v>
+          <t xml:space="preserve">cupom porcentagem</t>
+        </is>
+      </c>
+      <c r="B73" s="56">
+        <v>0.3</v>
+      </c>
+      <c t="inlineStr" r="C73">
+        <is>
+          <t xml:space="preserve">desconto30</t>
+        </is>
+      </c>
+      <c t="n" r="D73">
+        <v>11</v>
       </c>
       <c t="n" r="E73">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c t="inlineStr" r="F73">
         <is>
@@ -2754,17 +2753,22 @@
     <row r="74">
       <c t="inlineStr" r="A74">
         <is>
-          <t xml:space="preserve">Teste 21013</t>
+          <t xml:space="preserve">cupom3030desconto</t>
         </is>
       </c>
       <c r="B74" s="56">
-        <v>0.5</v>
-      </c>
-      <c r="C74" s="65">
-        <v>21013</v>
+        <v>0.3</v>
+      </c>
+      <c t="inlineStr" r="C74">
+        <is>
+          <t xml:space="preserve">desconto30%</t>
+        </is>
+      </c>
+      <c t="n" r="D74">
+        <v>11</v>
       </c>
       <c t="n" r="E74">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c t="inlineStr" r="F74">
         <is>
@@ -2785,31 +2789,28 @@
     <row r="75">
       <c t="inlineStr" r="A75">
         <is>
-          <t xml:space="preserve">cupom teste 21/01</t>
-        </is>
-      </c>
-      <c r="B75" s="56">
-        <v>0.3</v>
-      </c>
-      <c t="inlineStr" r="C75">
-        <is>
-          <t xml:space="preserve">my20261</t>
-        </is>
-      </c>
-      <c t="n" r="D75">
-        <v>11</v>
+          <t xml:space="preserve">Teste Metade 1</t>
+        </is>
+      </c>
+      <c t="inlineStr" r="B75">
+        <is>
+          <t xml:space="preserve">R$ 1.00</t>
+        </is>
+      </c>
+      <c r="C75" s="65">
+        <v>2201</v>
       </c>
       <c t="n" r="E75">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c t="inlineStr" r="F75">
         <is>
-          <t xml:space="preserve">21/01/2026 13:00:00</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c t="inlineStr" r="G75">
         <is>
-          <t xml:space="preserve">21/01/2026 13:25:00</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c t="inlineStr" r="H75">
@@ -2821,22 +2822,17 @@
     <row r="76">
       <c t="inlineStr" r="A76">
         <is>
-          <t xml:space="preserve">cupom porcentagem</t>
+          <t xml:space="preserve">Valor Minimo 2</t>
         </is>
       </c>
       <c r="B76" s="56">
-        <v>0.3</v>
-      </c>
-      <c t="inlineStr" r="C76">
-        <is>
-          <t xml:space="preserve">desconto30</t>
-        </is>
-      </c>
-      <c t="n" r="D76">
-        <v>11</v>
+        <v>0.01</v>
+      </c>
+      <c r="C76" s="65">
+        <v>2203</v>
       </c>
       <c t="n" r="E76">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c t="inlineStr" r="F76">
         <is>
@@ -2850,29 +2846,24 @@
       </c>
       <c t="inlineStr" r="H76">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">R$ 3.00</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c t="inlineStr" r="A77">
         <is>
-          <t xml:space="preserve">cupom3030desconto</t>
+          <t xml:space="preserve">teste</t>
         </is>
       </c>
       <c r="B77" s="56">
-        <v>0.3</v>
-      </c>
-      <c t="inlineStr" r="C77">
-        <is>
-          <t xml:space="preserve">desconto30%</t>
-        </is>
-      </c>
-      <c t="n" r="D77">
-        <v>11</v>
+        <v>0.5</v>
+      </c>
+      <c r="C77" s="65">
+        <v>5656</v>
       </c>
       <c t="n" r="E77">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c t="inlineStr" r="F77">
         <is>
@@ -2891,52 +2882,54 @@
       </c>
     </row>
     <row r="78">
-      <c t="inlineStr" r="A78">
-        <is>
-          <t xml:space="preserve">Teste Metade 1</t>
-        </is>
-      </c>
-      <c t="inlineStr" r="B78">
-        <is>
-          <t xml:space="preserve">R$ 1.00</t>
-        </is>
+      <c r="A78" s="65">
+        <v>2601</v>
+      </c>
+      <c r="B78" s="56">
+        <v>0.5</v>
       </c>
       <c r="C78" s="65">
-        <v>2201</v>
+        <v>2601</v>
+      </c>
+      <c t="n" r="D78">
+        <v>1</v>
       </c>
       <c t="n" r="E78">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c t="inlineStr" r="F78">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">26/01/2026 11:00:00</t>
         </is>
       </c>
       <c t="inlineStr" r="G78">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">26/01/2026 12:00:00</t>
         </is>
       </c>
       <c t="inlineStr" r="H78">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">R$ 2.00</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c t="inlineStr" r="A79">
         <is>
-          <t xml:space="preserve">Valor Minimo 2</t>
+          <t xml:space="preserve">2601-1</t>
         </is>
       </c>
       <c r="B79" s="56">
-        <v>0.01</v>
+        <v>0.5</v>
       </c>
       <c r="C79" s="65">
-        <v>2203</v>
+        <v>26011</v>
+      </c>
+      <c t="n" r="D79">
+        <v>1</v>
       </c>
       <c t="n" r="E79">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c t="inlineStr" r="F79">
         <is>
@@ -2950,33 +2943,33 @@
       </c>
       <c t="inlineStr" r="H79">
         <is>
-          <t xml:space="preserve">R$ 3.00</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c t="inlineStr" r="A80">
         <is>
-          <t xml:space="preserve">teste</t>
+          <t xml:space="preserve">2601-2</t>
         </is>
       </c>
       <c r="B80" s="56">
-        <v>0.5</v>
+        <v>260.12</v>
       </c>
       <c r="C80" s="65">
-        <v>5656</v>
+        <v>26012</v>
       </c>
       <c t="n" r="E80">
         <v>0</v>
       </c>
       <c t="inlineStr" r="F80">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">26/01/2026 00:00:00</t>
         </is>
       </c>
       <c t="inlineStr" r="G80">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">26/01/2026 11:10:00</t>
         </is>
       </c>
       <c t="inlineStr" r="H80">
@@ -2987,62 +2980,63 @@
     </row>
     <row r="81">
       <c r="A81" s="65">
-        <v>2601</v>
-      </c>
-      <c r="B81" s="56">
-        <v>0.5</v>
+        <v>26013</v>
+      </c>
+      <c t="inlineStr" r="B81">
+        <is>
+          <t xml:space="preserve">R$ 1.00</t>
+        </is>
       </c>
       <c r="C81" s="65">
-        <v>2601</v>
-      </c>
-      <c t="n" r="D81">
-        <v>1</v>
+        <v>26013</v>
       </c>
       <c t="n" r="E81">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c t="inlineStr" r="F81">
         <is>
-          <t xml:space="preserve">26/01/2026 11:00:00</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c t="inlineStr" r="G81">
         <is>
-          <t xml:space="preserve">26/01/2026 12:00:00</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c t="inlineStr" r="H81">
         <is>
-          <t xml:space="preserve">R$ 2.00</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c t="inlineStr" r="A82">
         <is>
-          <t xml:space="preserve">2601-1</t>
+          <t xml:space="preserve">cupom 27/01 checklist</t>
         </is>
       </c>
       <c r="B82" s="56">
-        <v>0.5</v>
-      </c>
-      <c r="C82" s="65">
-        <v>26011</v>
+        <v>0.3</v>
+      </c>
+      <c t="inlineStr" r="C82">
+        <is>
+          <t xml:space="preserve">semogoiac</t>
+        </is>
       </c>
       <c t="n" r="D82">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c t="n" r="E82">
         <v>1</v>
       </c>
       <c t="inlineStr" r="F82">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">27/01/2026 11:10:00</t>
         </is>
       </c>
       <c t="inlineStr" r="G82">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">27/01/2026 11:15:00</t>
         </is>
       </c>
       <c t="inlineStr" r="H82">
@@ -3054,26 +3048,28 @@
     <row r="83">
       <c t="inlineStr" r="A83">
         <is>
-          <t xml:space="preserve">2601-2</t>
+          <t xml:space="preserve">LECTOR10</t>
         </is>
       </c>
       <c r="B83" s="56">
-        <v>260.12</v>
-      </c>
-      <c r="C83" s="65">
-        <v>26012</v>
+        <v>0.5</v>
+      </c>
+      <c t="inlineStr" r="C83">
+        <is>
+          <t xml:space="preserve">LECTOR10</t>
+        </is>
       </c>
       <c t="n" r="E83">
         <v>0</v>
       </c>
       <c t="inlineStr" r="F83">
         <is>
-          <t xml:space="preserve">26/01/2026 00:00:00</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c t="inlineStr" r="G83">
         <is>
-          <t xml:space="preserve">26/01/2026 11:10:00</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c t="inlineStr" r="H83">
@@ -3083,64 +3079,69 @@
       </c>
     </row>
     <row r="84">
-      <c r="A84" s="65">
-        <v>26013</v>
-      </c>
-      <c t="inlineStr" r="B84">
-        <is>
-          <t xml:space="preserve">R$ 1.00</t>
-        </is>
-      </c>
-      <c r="C84" s="65">
-        <v>26013</v>
+      <c t="inlineStr" r="A84">
+        <is>
+          <t xml:space="preserve">0602 Teste</t>
+        </is>
+      </c>
+      <c r="B84" s="56">
+        <v>0.5</v>
+      </c>
+      <c t="inlineStr" r="C84">
+        <is>
+          <t xml:space="preserve">0602</t>
+        </is>
+      </c>
+      <c t="n" r="D84">
+        <v>1</v>
       </c>
       <c t="n" r="E84">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c t="inlineStr" r="F84">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">06/02/2026 11:50:00</t>
         </is>
       </c>
       <c t="inlineStr" r="G84">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">06/02/2026 11:55:00</t>
         </is>
       </c>
       <c t="inlineStr" r="H84">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">R$ 2.00</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c t="inlineStr" r="A85">
         <is>
-          <t xml:space="preserve">cupom 27/01 checklist</t>
+          <t xml:space="preserve">Teste 0602</t>
         </is>
       </c>
       <c r="B85" s="56">
-        <v>0.3</v>
+        <v>0.5</v>
       </c>
       <c t="inlineStr" r="C85">
         <is>
-          <t xml:space="preserve">semogoiac</t>
+          <t xml:space="preserve">0602-1</t>
         </is>
       </c>
       <c t="n" r="D85">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c t="n" r="E85">
         <v>1</v>
       </c>
       <c t="inlineStr" r="F85">
         <is>
-          <t xml:space="preserve">27/01/2026 11:10:00</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c t="inlineStr" r="G85">
         <is>
-          <t xml:space="preserve">27/01/2026 11:15:00</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c t="inlineStr" r="H85">
@@ -3152,19 +3153,21 @@
     <row r="86">
       <c t="inlineStr" r="A86">
         <is>
-          <t xml:space="preserve">LECTOR10</t>
-        </is>
-      </c>
-      <c r="B86" s="56">
-        <v>0.5</v>
+          <t xml:space="preserve">0602-1</t>
+        </is>
+      </c>
+      <c t="inlineStr" r="B86">
+        <is>
+          <t xml:space="preserve">R$ 1.00</t>
+        </is>
       </c>
       <c t="inlineStr" r="C86">
         <is>
-          <t xml:space="preserve">LECTOR10</t>
+          <t xml:space="preserve">0602-3</t>
         </is>
       </c>
       <c t="n" r="E86">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c t="inlineStr" r="F86">
         <is>
@@ -3185,52 +3188,50 @@
     <row r="87">
       <c t="inlineStr" r="A87">
         <is>
-          <t xml:space="preserve">0602 Teste</t>
+          <t xml:space="preserve">cupomluiz</t>
         </is>
       </c>
       <c r="B87" s="56">
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c t="inlineStr" r="C87">
         <is>
-          <t xml:space="preserve">0602</t>
+          <t xml:space="preserve">luiz100</t>
         </is>
       </c>
       <c t="n" r="D87">
-        <v>1</v>
+        <v>100</v>
       </c>
       <c t="n" r="E87">
-        <v>0</v>
+        <v>11</v>
       </c>
       <c t="inlineStr" r="F87">
         <is>
-          <t xml:space="preserve">06/02/2026 11:50:00</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c t="inlineStr" r="G87">
         <is>
-          <t xml:space="preserve">06/02/2026 11:55:00</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c t="inlineStr" r="H87">
         <is>
-          <t xml:space="preserve">R$ 2.00</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c t="inlineStr" r="A88">
         <is>
-          <t xml:space="preserve">Teste 0602</t>
+          <t xml:space="preserve">teste</t>
         </is>
       </c>
       <c r="B88" s="56">
         <v>0.5</v>
       </c>
-      <c t="inlineStr" r="C88">
-        <is>
-          <t xml:space="preserve">0602-1</t>
-        </is>
+      <c r="C88" s="65">
+        <v>1602</v>
       </c>
       <c t="n" r="D88">
         <v>1</v>
@@ -3257,30 +3258,29 @@
     <row r="89">
       <c t="inlineStr" r="A89">
         <is>
-          <t xml:space="preserve">0602-1</t>
-        </is>
-      </c>
-      <c t="inlineStr" r="B89">
-        <is>
-          <t xml:space="preserve">R$ 1.00</t>
-        </is>
-      </c>
-      <c t="inlineStr" r="C89">
-        <is>
-          <t xml:space="preserve">0602-3</t>
-        </is>
+          <t xml:space="preserve">Teste 1602</t>
+        </is>
+      </c>
+      <c r="B89" s="56">
+        <v>0.5</v>
+      </c>
+      <c r="C89" s="65">
+        <v>16021</v>
+      </c>
+      <c t="n" r="D89">
+        <v>1</v>
       </c>
       <c t="n" r="E89">
         <v>1</v>
       </c>
       <c t="inlineStr" r="F89">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">16/02/2026 17:00:00</t>
         </is>
       </c>
       <c t="inlineStr" r="G89">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">16/02/2026 23:00:00</t>
         </is>
       </c>
       <c t="inlineStr" r="H89">
@@ -3292,22 +3292,19 @@
     <row r="90">
       <c t="inlineStr" r="A90">
         <is>
-          <t xml:space="preserve">cupomluiz</t>
-        </is>
-      </c>
-      <c r="B90" s="56">
-        <v>1</v>
-      </c>
-      <c t="inlineStr" r="C90">
-        <is>
-          <t xml:space="preserve">luiz100</t>
-        </is>
-      </c>
-      <c t="n" r="D90">
-        <v>100</v>
+          <t xml:space="preserve">Teste 1602 2</t>
+        </is>
+      </c>
+      <c t="inlineStr" r="B90">
+        <is>
+          <t xml:space="preserve">R$ 1.00</t>
+        </is>
+      </c>
+      <c r="C90" s="65">
+        <v>16022</v>
       </c>
       <c t="n" r="E90">
-        <v>11</v>
+        <v>2</v>
       </c>
       <c t="inlineStr" r="F90">
         <is>
@@ -3328,17 +3325,16 @@
     <row r="91">
       <c t="inlineStr" r="A91">
         <is>
-          <t xml:space="preserve">teste</t>
+          <t xml:space="preserve">teste cupom</t>
         </is>
       </c>
       <c r="B91" s="56">
-        <v>0.5</v>
-      </c>
-      <c r="C91" s="65">
-        <v>1602</v>
-      </c>
-      <c t="n" r="D91">
-        <v>1</v>
+        <v>0.11</v>
+      </c>
+      <c t="inlineStr" r="C91">
+        <is>
+          <t xml:space="preserve">codigo10teste</t>
+        </is>
       </c>
       <c t="n" r="E91">
         <v>1</v>
@@ -3362,62 +3358,66 @@
     <row r="92">
       <c t="inlineStr" r="A92">
         <is>
-          <t xml:space="preserve">Teste 1602</t>
-        </is>
-      </c>
-      <c r="B92" s="56">
-        <v>0.5</v>
+          <t xml:space="preserve">Valor Minimo 3</t>
+        </is>
+      </c>
+      <c t="inlineStr" r="B92">
+        <is>
+          <t xml:space="preserve">R$ 1.00</t>
+        </is>
       </c>
       <c r="C92" s="65">
-        <v>16021</v>
-      </c>
-      <c t="n" r="D92">
-        <v>1</v>
+        <v>1901</v>
       </c>
       <c t="n" r="E92">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c t="inlineStr" r="F92">
         <is>
-          <t xml:space="preserve">16/02/2026 17:00:00</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c t="inlineStr" r="G92">
         <is>
-          <t xml:space="preserve">16/02/2026 23:00:00</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c t="inlineStr" r="H92">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">R$ 100.00</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c t="inlineStr" r="A93">
         <is>
-          <t xml:space="preserve">Teste 1602 2</t>
+          <t xml:space="preserve">cupom10trilha</t>
         </is>
       </c>
       <c t="inlineStr" r="B93">
         <is>
-          <t xml:space="preserve">R$ 1.00</t>
-        </is>
-      </c>
-      <c r="C93" s="65">
-        <v>16022</v>
+          <t xml:space="preserve">R$ 10.00</t>
+        </is>
+      </c>
+      <c t="inlineStr" r="C93">
+        <is>
+          <t xml:space="preserve">cupom10trilha</t>
+        </is>
+      </c>
+      <c t="n" r="D93">
+        <v>5</v>
       </c>
       <c t="n" r="E93">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c t="inlineStr" r="F93">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">23/02/2026 17:00:00</t>
         </is>
       </c>
       <c t="inlineStr" r="G93">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">23/02/2026 17:55:00</t>
         </is>
       </c>
       <c t="inlineStr" r="H93">
@@ -3429,19 +3429,19 @@
     <row r="94">
       <c t="inlineStr" r="A94">
         <is>
-          <t xml:space="preserve">teste cupom</t>
-        </is>
-      </c>
-      <c r="B94" s="56">
-        <v>0.11</v>
-      </c>
-      <c t="inlineStr" r="C94">
-        <is>
-          <t xml:space="preserve">codigo10teste</t>
-        </is>
+          <t xml:space="preserve">Teste100</t>
+        </is>
+      </c>
+      <c t="inlineStr" r="B94">
+        <is>
+          <t xml:space="preserve">R$ 1.00</t>
+        </is>
+      </c>
+      <c r="C94" s="65">
+        <v>99</v>
       </c>
       <c t="n" r="E94">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c t="inlineStr" r="F94">
         <is>
@@ -3462,29 +3462,26 @@
     <row r="95">
       <c t="inlineStr" r="A95">
         <is>
-          <t xml:space="preserve">Cupom Cypress</t>
+          <t xml:space="preserve">Teste 200</t>
         </is>
       </c>
       <c r="B95" s="56">
         <v>0.5</v>
       </c>
       <c r="C95" s="65">
-        <v>808182</v>
-      </c>
-      <c t="n" r="D95">
-        <v>80</v>
+        <v>88</v>
       </c>
       <c t="n" r="E95">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c t="inlineStr" r="F95">
         <is>
-          <t xml:space="preserve">01/01/2026 10:00:00</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c t="inlineStr" r="G95">
         <is>
-          <t xml:space="preserve">05/12/2026 18:00:00</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c t="inlineStr" r="H95">
@@ -3496,66 +3493,57 @@
     <row r="96">
       <c t="inlineStr" r="A96">
         <is>
-          <t xml:space="preserve">Valor Minimo 3</t>
-        </is>
-      </c>
-      <c t="inlineStr" r="B96">
-        <is>
-          <t xml:space="preserve">R$ 1.00</t>
-        </is>
+          <t xml:space="preserve">expirado</t>
+        </is>
+      </c>
+      <c r="B96" s="56">
+        <v>0.5</v>
       </c>
       <c r="C96" s="65">
-        <v>1901</v>
+        <v>77</v>
       </c>
       <c t="n" r="E96">
         <v>0</v>
       </c>
       <c t="inlineStr" r="F96">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">24/02/2026 10:00:00</t>
         </is>
       </c>
       <c t="inlineStr" r="G96">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">24/02/2026 10:10:00</t>
         </is>
       </c>
       <c t="inlineStr" r="H96">
         <is>
-          <t xml:space="preserve">R$ 100.00</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
     </row>
     <row r="97">
       <c t="inlineStr" r="A97">
         <is>
-          <t xml:space="preserve">cupom10trilha</t>
-        </is>
-      </c>
-      <c t="inlineStr" r="B97">
-        <is>
-          <t xml:space="preserve">R$ 10.00</t>
-        </is>
-      </c>
-      <c t="inlineStr" r="C97">
-        <is>
-          <t xml:space="preserve">cupom10trilha</t>
-        </is>
-      </c>
-      <c t="n" r="D97">
-        <v>5</v>
+          <t xml:space="preserve">teste 3</t>
+        </is>
+      </c>
+      <c r="B97" s="56">
+        <v>0.5</v>
+      </c>
+      <c r="C97" s="65">
+        <v>55</v>
       </c>
       <c t="n" r="E97">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c t="inlineStr" r="F97">
         <is>
-          <t xml:space="preserve">23/02/2026 17:00:00</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c t="inlineStr" r="G97">
         <is>
-          <t xml:space="preserve">23/02/2026 17:55:00</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c t="inlineStr" r="H97">
@@ -3567,7 +3555,7 @@
     <row r="98">
       <c t="inlineStr" r="A98">
         <is>
-          <t xml:space="preserve">Teste100</t>
+          <t xml:space="preserve">teste 1</t>
         </is>
       </c>
       <c t="inlineStr" r="B98">
@@ -3576,10 +3564,13 @@
         </is>
       </c>
       <c r="C98" s="65">
-        <v>99</v>
+        <v>44</v>
+      </c>
+      <c t="n" r="D98">
+        <v>1</v>
       </c>
       <c t="n" r="E98">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c t="inlineStr" r="F98">
         <is>
@@ -3600,17 +3591,19 @@
     <row r="99">
       <c t="inlineStr" r="A99">
         <is>
-          <t xml:space="preserve">Teste 200</t>
-        </is>
-      </c>
-      <c r="B99" s="56">
-        <v>0.5</v>
+          <t xml:space="preserve">Vencido</t>
+        </is>
+      </c>
+      <c t="inlineStr" r="B99">
+        <is>
+          <t xml:space="preserve">R$ 1.00</t>
+        </is>
       </c>
       <c r="C99" s="65">
-        <v>88</v>
+        <v>202020</v>
       </c>
       <c t="n" r="E99">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c t="inlineStr" r="F99">
         <is>
@@ -3631,26 +3624,28 @@
     <row r="100">
       <c t="inlineStr" r="A100">
         <is>
-          <t xml:space="preserve">expirado</t>
-        </is>
-      </c>
-      <c r="B100" s="56">
-        <v>0.5</v>
+          <t xml:space="preserve">Real 1</t>
+        </is>
+      </c>
+      <c t="inlineStr" r="B100">
+        <is>
+          <t xml:space="preserve">R$ 1.00</t>
+        </is>
       </c>
       <c r="C100" s="65">
-        <v>77</v>
+        <v>303030</v>
       </c>
       <c t="n" r="E100">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c t="inlineStr" r="F100">
         <is>
-          <t xml:space="preserve">24/02/2026 10:00:00</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c t="inlineStr" r="G100">
         <is>
-          <t xml:space="preserve">24/02/2026 10:10:00</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c t="inlineStr" r="H100">
@@ -3662,17 +3657,22 @@
     <row r="101">
       <c t="inlineStr" r="A101">
         <is>
-          <t xml:space="preserve">teste 3</t>
-        </is>
-      </c>
-      <c r="B101" s="56">
-        <v>0.5</v>
+          <t xml:space="preserve">Real 2</t>
+        </is>
+      </c>
+      <c t="inlineStr" r="B101">
+        <is>
+          <t xml:space="preserve">R$ 1.00</t>
+        </is>
       </c>
       <c r="C101" s="65">
-        <v>55</v>
+        <v>404040</v>
+      </c>
+      <c t="n" r="D101">
+        <v>1</v>
       </c>
       <c t="n" r="E101">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c t="inlineStr" r="F101">
         <is>
@@ -3693,19 +3693,14 @@
     <row r="102">
       <c t="inlineStr" r="A102">
         <is>
-          <t xml:space="preserve">teste 1</t>
-        </is>
-      </c>
-      <c t="inlineStr" r="B102">
-        <is>
-          <t xml:space="preserve">R$ 1.00</t>
-        </is>
+          <t xml:space="preserve">Porcentagem</t>
+        </is>
+      </c>
+      <c r="B102" s="56">
+        <v>0.5</v>
       </c>
       <c r="C102" s="65">
-        <v>44</v>
-      </c>
-      <c t="n" r="D102">
-        <v>1</v>
+        <v>707070</v>
       </c>
       <c t="n" r="E102">
         <v>1</v>
@@ -3729,19 +3724,17 @@
     <row r="103">
       <c t="inlineStr" r="A103">
         <is>
-          <t xml:space="preserve">Vencido</t>
-        </is>
-      </c>
-      <c t="inlineStr" r="B103">
-        <is>
-          <t xml:space="preserve">R$ 1.00</t>
-        </is>
+          <t xml:space="preserve">Valor minimo</t>
+        </is>
+      </c>
+      <c r="B103" s="56">
+        <v>0.5</v>
       </c>
       <c r="C103" s="65">
-        <v>202020</v>
+        <v>909090</v>
       </c>
       <c t="n" r="E103">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c t="inlineStr" r="F103">
         <is>
@@ -3755,14 +3748,14 @@
       </c>
       <c t="inlineStr" r="H103">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">R$ 5.00</t>
         </is>
       </c>
     </row>
     <row r="104">
       <c t="inlineStr" r="A104">
         <is>
-          <t xml:space="preserve">Real 1</t>
+          <t xml:space="preserve">teste ext</t>
         </is>
       </c>
       <c t="inlineStr" r="B104">
@@ -3771,19 +3764,19 @@
         </is>
       </c>
       <c r="C104" s="65">
-        <v>303030</v>
+        <v>959595</v>
       </c>
       <c t="n" r="E104">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c t="inlineStr" r="F104">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">26/02/2026 09:00:00</t>
         </is>
       </c>
       <c t="inlineStr" r="G104">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">26/02/2026 09:20:00</t>
         </is>
       </c>
       <c t="inlineStr" r="H104">
@@ -3795,7 +3788,7 @@
     <row r="105">
       <c t="inlineStr" r="A105">
         <is>
-          <t xml:space="preserve">Real 2</t>
+          <t xml:space="preserve">teste 03</t>
         </is>
       </c>
       <c t="inlineStr" r="B105">
@@ -3803,8 +3796,10 @@
           <t xml:space="preserve">R$ 1.00</t>
         </is>
       </c>
-      <c r="C105" s="65">
-        <v>404040</v>
+      <c t="inlineStr" r="C105">
+        <is>
+          <t xml:space="preserve">0303</t>
+        </is>
       </c>
       <c t="n" r="D105">
         <v>1</v>
@@ -3814,43 +3809,43 @@
       </c>
       <c t="inlineStr" r="F105">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">03/03/2026 13:40:00</t>
         </is>
       </c>
       <c t="inlineStr" r="G105">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">03/03/2026 14:00:00</t>
         </is>
       </c>
       <c t="inlineStr" r="H105">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">R$ 1.00</t>
         </is>
       </c>
     </row>
     <row r="106">
       <c t="inlineStr" r="A106">
         <is>
-          <t xml:space="preserve">Porcentagem</t>
+          <t xml:space="preserve">expirado</t>
         </is>
       </c>
       <c r="B106" s="56">
         <v>0.5</v>
       </c>
       <c r="C106" s="65">
-        <v>707070</v>
+        <v>330</v>
       </c>
       <c t="n" r="E106">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c t="inlineStr" r="F106">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">03/03/2026 13:35:00</t>
         </is>
       </c>
       <c t="inlineStr" r="G106">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">03/03/2026 13:40:00</t>
         </is>
       </c>
       <c t="inlineStr" r="H106">
@@ -3862,14 +3857,14 @@
     <row r="107">
       <c t="inlineStr" r="A107">
         <is>
-          <t xml:space="preserve">Valor minimo</t>
+          <t xml:space="preserve">teste trilha</t>
         </is>
       </c>
       <c r="B107" s="56">
         <v>0.5</v>
       </c>
       <c r="C107" s="65">
-        <v>909090</v>
+        <v>61615</v>
       </c>
       <c t="n" r="E107">
         <v>0</v>
@@ -3886,35 +3881,33 @@
       </c>
       <c t="inlineStr" r="H107">
         <is>
-          <t xml:space="preserve">R$ 5.00</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
     </row>
     <row r="108">
       <c t="inlineStr" r="A108">
         <is>
-          <t xml:space="preserve">teste ext</t>
-        </is>
-      </c>
-      <c t="inlineStr" r="B108">
-        <is>
-          <t xml:space="preserve">R$ 1.00</t>
-        </is>
+          <t xml:space="preserve">teste</t>
+        </is>
+      </c>
+      <c r="B108" s="56">
+        <v>0.5</v>
       </c>
       <c r="C108" s="65">
-        <v>959595</v>
+        <v>61617</v>
       </c>
       <c t="n" r="E108">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c t="inlineStr" r="F108">
         <is>
-          <t xml:space="preserve">26/02/2026 09:00:00</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c t="inlineStr" r="G108">
         <is>
-          <t xml:space="preserve">26/02/2026 09:20:00</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c t="inlineStr" r="H108">
@@ -3926,7 +3919,7 @@
     <row r="109">
       <c t="inlineStr" r="A109">
         <is>
-          <t xml:space="preserve">teste 03</t>
+          <t xml:space="preserve">cupom teste 12</t>
         </is>
       </c>
       <c t="inlineStr" r="B109">
@@ -3934,56 +3927,54 @@
           <t xml:space="preserve">R$ 1.00</t>
         </is>
       </c>
-      <c t="inlineStr" r="C109">
-        <is>
-          <t xml:space="preserve">0303</t>
-        </is>
-      </c>
-      <c t="n" r="D109">
-        <v>1</v>
+      <c r="C109" s="65">
+        <v>1203</v>
       </c>
       <c t="n" r="E109">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c t="inlineStr" r="F109">
         <is>
-          <t xml:space="preserve">03/03/2026 13:40:00</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c t="inlineStr" r="G109">
         <is>
-          <t xml:space="preserve">03/03/2026 14:00:00</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c t="inlineStr" r="H109">
         <is>
-          <t xml:space="preserve">R$ 1.00</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
     </row>
     <row r="110">
       <c t="inlineStr" r="A110">
         <is>
-          <t xml:space="preserve">expirado</t>
+          <t xml:space="preserve">cupom teste 13</t>
         </is>
       </c>
       <c r="B110" s="56">
         <v>0.5</v>
       </c>
       <c r="C110" s="65">
-        <v>330</v>
+        <v>1204</v>
+      </c>
+      <c t="n" r="D110">
+        <v>1</v>
       </c>
       <c t="n" r="E110">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c t="inlineStr" r="F110">
         <is>
-          <t xml:space="preserve">03/03/2026 13:35:00</t>
+          <t xml:space="preserve">12/03/2026 08:45:00</t>
         </is>
       </c>
       <c t="inlineStr" r="G110">
         <is>
-          <t xml:space="preserve">03/03/2026 13:40:00</t>
+          <t xml:space="preserve">12/03/2026 09:30:00</t>
         </is>
       </c>
       <c t="inlineStr" r="H110">
@@ -3995,17 +3986,17 @@
     <row r="111">
       <c t="inlineStr" r="A111">
         <is>
-          <t xml:space="preserve">teste trilha</t>
+          <t xml:space="preserve">teste</t>
         </is>
       </c>
       <c r="B111" s="56">
         <v>0.5</v>
       </c>
       <c r="C111" s="65">
-        <v>61615</v>
+        <v>1205</v>
       </c>
       <c t="n" r="E111">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c t="inlineStr" r="F111">
         <is>
@@ -4026,17 +4017,17 @@
     <row r="112">
       <c t="inlineStr" r="A112">
         <is>
-          <t xml:space="preserve">teste</t>
+          <t xml:space="preserve">100% Teste</t>
         </is>
       </c>
       <c r="B112" s="56">
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="C112" s="65">
-        <v>61617</v>
+        <v>13033</v>
       </c>
       <c t="n" r="E112">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c t="inlineStr" r="F112">
         <is>
@@ -4057,7 +4048,7 @@
     <row r="113">
       <c t="inlineStr" r="A113">
         <is>
-          <t xml:space="preserve">cupom teste 12</t>
+          <t xml:space="preserve">Teste 1703</t>
         </is>
       </c>
       <c t="inlineStr" r="B113">
@@ -4066,53 +4057,53 @@
         </is>
       </c>
       <c r="C113" s="65">
-        <v>1203</v>
+        <v>17031</v>
+      </c>
+      <c t="n" r="D113">
+        <v>1</v>
       </c>
       <c t="n" r="E113">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c t="inlineStr" r="F113">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">17/03/2026 00:00:00</t>
         </is>
       </c>
       <c t="inlineStr" r="G113">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">18/03/2026 00:00:00</t>
         </is>
       </c>
       <c t="inlineStr" r="H113">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">R$ 2.00</t>
         </is>
       </c>
     </row>
     <row r="114">
       <c t="inlineStr" r="A114">
         <is>
-          <t xml:space="preserve">cupom teste 13</t>
+          <t xml:space="preserve">Teste 2 1703 expirado</t>
         </is>
       </c>
       <c r="B114" s="56">
-        <v>0.5</v>
+        <v>5</v>
       </c>
       <c r="C114" s="65">
-        <v>1204</v>
-      </c>
-      <c t="n" r="D114">
-        <v>1</v>
+        <v>17032</v>
       </c>
       <c t="n" r="E114">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c t="inlineStr" r="F114">
         <is>
-          <t xml:space="preserve">12/03/2026 08:45:00</t>
+          <t xml:space="preserve">17/03/2026 00:00:00</t>
         </is>
       </c>
       <c t="inlineStr" r="G114">
         <is>
-          <t xml:space="preserve">12/03/2026 09:30:00</t>
+          <t xml:space="preserve">17/03/2026 11:00:00</t>
         </is>
       </c>
       <c t="inlineStr" r="H114">
@@ -4124,17 +4115,17 @@
     <row r="115">
       <c t="inlineStr" r="A115">
         <is>
-          <t xml:space="preserve">teste</t>
+          <t xml:space="preserve">Teste3 1703</t>
         </is>
       </c>
       <c r="B115" s="56">
         <v>0.5</v>
       </c>
       <c r="C115" s="65">
-        <v>1205</v>
+        <v>17033</v>
       </c>
       <c t="n" r="E115">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c t="inlineStr" r="F115">
         <is>
@@ -4155,17 +4146,17 @@
     <row r="116">
       <c t="inlineStr" r="A116">
         <is>
-          <t xml:space="preserve">100% Teste</t>
+          <t xml:space="preserve">ValorAcimaDoMinimo2</t>
         </is>
       </c>
       <c r="B116" s="56">
-        <v>1</v>
+        <v>0.5</v>
       </c>
       <c r="C116" s="65">
-        <v>13033</v>
+        <v>919293</v>
       </c>
       <c t="n" r="E116">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c t="inlineStr" r="F116">
         <is>
@@ -4179,15 +4170,13 @@
       </c>
       <c t="inlineStr" r="H116">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">R$ 50.00</t>
         </is>
       </c>
     </row>
     <row r="117">
-      <c t="inlineStr" r="A117">
-        <is>
-          <t xml:space="preserve">Teste 1703</t>
-        </is>
+      <c r="A117" s="65">
+        <v>777</v>
       </c>
       <c t="inlineStr" r="B117">
         <is>
@@ -4195,53 +4184,50 @@
         </is>
       </c>
       <c r="C117" s="65">
-        <v>17031</v>
-      </c>
-      <c t="n" r="D117">
-        <v>1</v>
+        <v>111225</v>
       </c>
       <c t="n" r="E117">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c t="inlineStr" r="F117">
         <is>
-          <t xml:space="preserve">17/03/2026 00:00:00</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c t="inlineStr" r="G117">
         <is>
-          <t xml:space="preserve">18/03/2026 00:00:00</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c t="inlineStr" r="H117">
         <is>
-          <t xml:space="preserve">R$ 2.00</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
     </row>
     <row r="118">
       <c t="inlineStr" r="A118">
         <is>
-          <t xml:space="preserve">Teste 2 1703 expirado</t>
+          <t xml:space="preserve">ok</t>
         </is>
       </c>
       <c r="B118" s="56">
-        <v>5</v>
+        <v>0.5</v>
       </c>
       <c r="C118" s="65">
-        <v>17032</v>
+        <v>2025</v>
       </c>
       <c t="n" r="E118">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c t="inlineStr" r="F118">
         <is>
-          <t xml:space="preserve">17/03/2026 00:00:00</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c t="inlineStr" r="G118">
         <is>
-          <t xml:space="preserve">17/03/2026 11:00:00</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c t="inlineStr" r="H118">
@@ -4253,17 +4239,17 @@
     <row r="119">
       <c t="inlineStr" r="A119">
         <is>
-          <t xml:space="preserve">Teste3 1703</t>
+          <t xml:space="preserve">porcetagem20</t>
         </is>
       </c>
       <c r="B119" s="56">
         <v>0.5</v>
       </c>
       <c r="C119" s="65">
-        <v>17033</v>
+        <v>200420</v>
       </c>
       <c t="n" r="E119">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c t="inlineStr" r="F119">
         <is>
@@ -4284,17 +4270,24 @@
     <row r="120">
       <c t="inlineStr" r="A120">
         <is>
-          <t xml:space="preserve">ValorAcimaDoMinimo2</t>
-        </is>
-      </c>
-      <c r="B120" s="56">
-        <v>0.5</v>
-      </c>
-      <c r="C120" s="65">
-        <v>919293</v>
+          <t xml:space="preserve">valor 102</t>
+        </is>
+      </c>
+      <c t="inlineStr" r="B120">
+        <is>
+          <t xml:space="preserve">R$ 1.00</t>
+        </is>
+      </c>
+      <c t="inlineStr" r="C120">
+        <is>
+          <t xml:space="preserve">045069</t>
+        </is>
+      </c>
+      <c t="n" r="D120">
+        <v>1</v>
       </c>
       <c t="n" r="E120">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c t="inlineStr" r="F120">
         <is>
@@ -4308,13 +4301,13 @@
       </c>
       <c t="inlineStr" r="H120">
         <is>
-          <t xml:space="preserve">R$ 50.00</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
     </row>
     <row r="121">
       <c r="A121" s="65">
-        <v>777</v>
+        <v>111</v>
       </c>
       <c t="inlineStr" r="B121">
         <is>
@@ -4322,7 +4315,7 @@
         </is>
       </c>
       <c r="C121" s="65">
-        <v>111225</v>
+        <v>1111111111</v>
       </c>
       <c t="n" r="E121">
         <v>0</v>
@@ -4338,6 +4331,35 @@
         </is>
       </c>
       <c t="inlineStr" r="H121">
+        <is>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" s="65">
+        <v>2222</v>
+      </c>
+      <c r="B122" s="56">
+        <v>22.22</v>
+      </c>
+      <c r="C122" s="65">
+        <v>222222</v>
+      </c>
+      <c t="n" r="E122">
+        <v>0</v>
+      </c>
+      <c t="inlineStr" r="F122">
+        <is>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+      <c t="inlineStr" r="G122">
+        <is>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+      <c t="inlineStr" r="H122">
         <is>
           <t xml:space="preserve">-</t>
         </is>

</xml_diff>